<commit_message>
Make Core the base product and add extra licenses
Every Core subscription includes 5 licenses (1 master + 4 dependents)
and each extra license is R$ 300/month. Sprint buyers get 1 month of
Core and Scale buyers 3 months; out-of-base Sprint buyers then become
Core subscribers (79 clients by month 24). Partner pay is recalibrated
to 3.5% each so break-even stays at month 6. VPL at 24% a.a. goes to
R$ 167,9 mil, TIR 126%. Form, workbooks, planning document, pitch slides
10/11/12/16 and the calculation memo are all regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016kLWp3PkVdryYcjkVkag3m
</commit_message>
<xml_diff>
--- a/precept-financeiro/Planilha_Financeira_Precept.xlsx
+++ b/precept-financeiro/Planilha_Financeira_Precept.xlsx
@@ -1305,24 +1305,24 @@
         <v>1</v>
       </c>
       <c r="B6" s="11" t="n">
-        <v>4788</v>
+        <v>5988</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>1197.9</v>
+        <v>1479.9</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>12000</v>
       </c>
       <c r="E6" s="12" t="n">
         <f aca="false">B6-C6-D6</f>
-        <v>-8409.9</v>
+        <v>-7491.9</v>
       </c>
       <c r="F6" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="13" t="n">
         <f aca="false">E6-F6</f>
-        <v>-8409.9</v>
+        <v>-7491.9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1330,24 +1330,24 @@
         <v>2</v>
       </c>
       <c r="B7" s="11" t="n">
-        <v>7182</v>
+        <v>8982</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>1796.85</v>
+        <v>2219.85</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>12000</v>
       </c>
       <c r="E7" s="12" t="n">
         <f aca="false">B7-C7-D7</f>
-        <v>-6614.85</v>
+        <v>-5237.85</v>
       </c>
       <c r="F7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="13" t="n">
         <f aca="false">E7-F7</f>
-        <v>-6614.85</v>
+        <v>-5237.85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1355,24 +1355,24 @@
         <v>3</v>
       </c>
       <c r="B8" s="11" t="n">
-        <v>10773</v>
+        <v>13473</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>2695.28</v>
+        <v>3329.78</v>
       </c>
       <c r="D8" s="11" t="n">
         <v>12000</v>
       </c>
       <c r="E8" s="12" t="n">
         <f aca="false">B8-C8-D8</f>
-        <v>-3922.28</v>
+        <v>-1856.78</v>
       </c>
       <c r="F8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="13" t="n">
         <f aca="false">E8-F8</f>
-        <v>-3922.28</v>
+        <v>-1856.78</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1380,24 +1380,24 @@
         <v>4</v>
       </c>
       <c r="B9" s="11" t="n">
-        <v>23164</v>
+        <v>24967</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>9642.5</v>
+        <v>10156.02</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>16864.44</v>
+        <v>18116.92</v>
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">B9-C9-D9</f>
-        <v>-3342.94</v>
+        <v>-3305.94</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="13" t="n">
         <f aca="false">E9-F9</f>
-        <v>-3342.94</v>
+        <v>-3305.94</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1405,24 +1405,24 @@
         <v>5</v>
       </c>
       <c r="B10" s="11" t="n">
-        <v>26755</v>
+        <v>29458</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>10540.92</v>
+        <v>11265.95</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>17618.55</v>
+        <v>19217.21</v>
       </c>
       <c r="E10" s="12" t="n">
         <f aca="false">B10-C10-D10</f>
-        <v>-1404.47</v>
+        <v>-1025.16</v>
       </c>
       <c r="F10" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="13" t="n">
         <f aca="false">E10-F10</f>
-        <v>-1404.47</v>
+        <v>-1025.16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1430,24 +1430,24 @@
         <v>6</v>
       </c>
       <c r="B11" s="11" t="n">
-        <v>34148.5</v>
+        <v>35954.5</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>14214.59</v>
+        <v>14903.98</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>19171.18</v>
+        <v>20808.85</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">B11-C11-D11</f>
-        <v>762.73</v>
+        <v>241.670000000002</v>
       </c>
       <c r="F11" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="13" t="n">
         <f aca="false">E11-F11</f>
-        <v>762.73</v>
+        <v>241.670000000002</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1455,24 +1455,24 @@
         <v>7</v>
       </c>
       <c r="B12" s="11" t="n">
-        <v>37739.5</v>
+        <v>40445.5</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>15261.5</v>
+        <v>16173.83</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>19925.29</v>
+        <v>21909.15</v>
       </c>
       <c r="E12" s="12" t="n">
         <f aca="false">B12-C12-D12</f>
-        <v>2552.71</v>
+        <v>2362.52</v>
       </c>
       <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="13" t="n">
         <f aca="false">E12-F12</f>
-        <v>2552.71</v>
+        <v>2362.52</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1480,24 +1480,24 @@
         <v>8</v>
       </c>
       <c r="B13" s="11" t="n">
-        <v>45133</v>
+        <v>46942</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>19095.39</v>
+        <v>19881.12</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>21477.93</v>
+        <v>23500.79</v>
       </c>
       <c r="E13" s="12" t="n">
         <f aca="false">B13-C13-D13</f>
-        <v>4559.68</v>
+        <v>3560.09</v>
       </c>
       <c r="F13" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">E13-F13</f>
-        <v>4559.68</v>
+        <v>3560.09</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1505,24 +1505,24 @@
         <v>9</v>
       </c>
       <c r="B14" s="11" t="n">
-        <v>58721</v>
+        <v>61430</v>
       </c>
       <c r="C14" s="11" t="n">
-        <v>26572.68</v>
+        <v>27581.5</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>24331.41</v>
+        <v>27050.35</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">B14-C14-D14</f>
-        <v>7816.91</v>
+        <v>6798.15</v>
       </c>
       <c r="F14" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">E14-F14</f>
-        <v>7816.91</v>
+        <v>6798.15</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1530,24 +1530,24 @@
         <v>10</v>
       </c>
       <c r="B15" s="11" t="n">
-        <v>56117.5</v>
+        <v>59426.5</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>23999.25</v>
+        <v>25142.12</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>23784.67</v>
+        <v>26559.49</v>
       </c>
       <c r="E15" s="12" t="n">
         <f aca="false">B15-C15-D15</f>
-        <v>8333.58</v>
+        <v>7724.89</v>
       </c>
       <c r="F15" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="13" t="n">
         <f aca="false">E15-F15</f>
-        <v>8333.58</v>
+        <v>7724.89</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1555,24 +1555,24 @@
         <v>11</v>
       </c>
       <c r="B16" s="11" t="n">
-        <v>69705.5</v>
+        <v>73914.5</v>
       </c>
       <c r="C16" s="11" t="n">
-        <v>31505.24</v>
+        <v>32956.18</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>26638.15</v>
+        <v>30109.05</v>
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">B16-C16-D16</f>
-        <v>11562.11</v>
+        <v>10849.27</v>
       </c>
       <c r="F16" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="13" t="n">
         <f aca="false">E16-F16</f>
-        <v>11562.11</v>
+        <v>10849.27</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1580,24 +1580,24 @@
         <v>12</v>
       </c>
       <c r="B17" s="11" t="n">
-        <v>62102.5</v>
+        <v>66911.5</v>
       </c>
       <c r="C17" s="11" t="n">
-        <v>25834.25</v>
+        <v>27417.83</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>25041.53</v>
+        <v>28393.32</v>
       </c>
       <c r="E17" s="12" t="n">
         <f aca="false">B17-C17-D17</f>
-        <v>11226.72</v>
+        <v>11100.35</v>
       </c>
       <c r="F17" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G17" s="13" t="n">
         <f aca="false">E17-F17</f>
-        <v>11226.72</v>
+        <v>11100.35</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1605,24 +1605,24 @@
         <v>13</v>
       </c>
       <c r="B18" s="11" t="n">
-        <v>100684</v>
+        <v>104896</v>
       </c>
       <c r="C18" s="11" t="n">
-        <v>49617.01</v>
+        <v>51415.58</v>
       </c>
       <c r="D18" s="11" t="n">
-        <v>33143.64</v>
+        <v>37699.52</v>
       </c>
       <c r="E18" s="12" t="n">
         <f aca="false">B18-C18-D18</f>
-        <v>17923.35</v>
+        <v>15780.9</v>
       </c>
       <c r="F18" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="13" t="n">
         <f aca="false">E18-F18</f>
-        <v>17923.35</v>
+        <v>15780.9</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1630,24 +1630,24 @@
         <v>14</v>
       </c>
       <c r="B19" s="11" t="n">
-        <v>103078</v>
+        <v>109387</v>
       </c>
       <c r="C19" s="11" t="n">
-        <v>50678.8</v>
+        <v>53122</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>33646.38</v>
+        <v>38799.82</v>
       </c>
       <c r="E19" s="12" t="n">
         <f aca="false">B19-C19-D19</f>
-        <v>18752.82</v>
+        <v>17465.18</v>
       </c>
       <c r="F19" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G19" s="13" t="n">
         <f aca="false">E19-F19</f>
-        <v>18752.82</v>
+        <v>17465.18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1655,24 +1655,24 @@
         <v>15</v>
       </c>
       <c r="B20" s="11" t="n">
-        <v>110471.5</v>
+        <v>120374.5</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>54824.4</v>
+        <v>58240.6</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>35199.01</v>
+        <v>41491.75</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">B20-C20-D20</f>
-        <v>20448.09</v>
+        <v>20642.15</v>
       </c>
       <c r="F20" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="13" t="n">
         <f aca="false">E20-F20</f>
-        <v>20448.09</v>
+        <v>20642.15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1680,24 +1680,24 @@
         <v>16</v>
       </c>
       <c r="B21" s="11" t="n">
-        <v>112865.5</v>
+        <v>126362.5</v>
       </c>
       <c r="C21" s="11" t="n">
-        <v>55737.18</v>
+        <v>60218.42</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>35701.75</v>
+        <v>42958.81</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">B21-C21-D21</f>
-        <v>21426.57</v>
+        <v>23185.27</v>
       </c>
       <c r="F21" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">E21-F21</f>
-        <v>21426.57</v>
+        <v>23185.27</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1705,24 +1705,24 @@
         <v>17</v>
       </c>
       <c r="B22" s="11" t="n">
-        <v>120259</v>
+        <v>135853</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>59916.83</v>
+        <v>65015.49</v>
       </c>
       <c r="D22" s="11" t="n">
-        <v>37254.39</v>
+        <v>45283.99</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">B22-C22-D22</f>
-        <v>23087.78</v>
+        <v>25553.52</v>
       </c>
       <c r="F22" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">E22-F22</f>
-        <v>23087.78</v>
+        <v>25553.52</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1730,24 +1730,24 @@
         <v>18</v>
       </c>
       <c r="B23" s="11" t="n">
-        <v>122653</v>
+        <v>141841</v>
       </c>
       <c r="C23" s="11" t="n">
-        <v>60848.72</v>
+        <v>66978.03</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>37757.13</v>
+        <v>46751.05</v>
       </c>
       <c r="E23" s="12" t="n">
         <f aca="false">B23-C23-D23</f>
-        <v>24047.15</v>
+        <v>28111.92</v>
       </c>
       <c r="F23" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">E23-F23</f>
-        <v>24047.15</v>
+        <v>28111.92</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1755,24 +1755,24 @@
         <v>19</v>
       </c>
       <c r="B24" s="11" t="n">
-        <v>135044</v>
+        <v>157826</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>68407.36</v>
+        <v>75702.62</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>40359.24</v>
+        <v>50667.37</v>
       </c>
       <c r="E24" s="12" t="n">
         <f aca="false">B24-C24-D24</f>
-        <v>26277.4</v>
+        <v>31456.01</v>
       </c>
       <c r="F24" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="13" t="n">
         <f aca="false">E24-F24</f>
-        <v>26277.4</v>
+        <v>31456.01</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1780,24 +1780,24 @@
         <v>20</v>
       </c>
       <c r="B25" s="11" t="n">
-        <v>137438</v>
+        <v>163814</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>69293.65</v>
+        <v>77638.6</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>40861.98</v>
+        <v>52134.43</v>
       </c>
       <c r="E25" s="12" t="n">
         <f aca="false">B25-C25-D25</f>
-        <v>27282.37</v>
+        <v>34040.97</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">E25-F25</f>
-        <v>27282.37</v>
+        <v>34040.97</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1805,24 +1805,24 @@
         <v>21</v>
       </c>
       <c r="B26" s="11" t="n">
-        <v>139832</v>
+        <v>169802</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>70144.2</v>
+        <v>79545.93</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>41364.72</v>
+        <v>53601.49</v>
       </c>
       <c r="E26" s="12" t="n">
         <f aca="false">B26-C26-D26</f>
-        <v>28323.08</v>
+        <v>36654.58</v>
       </c>
       <c r="F26" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="13" t="n">
         <f aca="false">E26-F26</f>
-        <v>28323.08</v>
+        <v>36654.58</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1830,24 +1830,24 @@
         <v>22</v>
       </c>
       <c r="B27" s="11" t="n">
-        <v>142226</v>
+        <v>174293</v>
       </c>
       <c r="C27" s="11" t="n">
-        <v>70959.02</v>
+        <v>80993.12</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>41867.46</v>
+        <v>54701.79</v>
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">B27-C27-D27</f>
-        <v>29399.52</v>
+        <v>38598.09</v>
       </c>
       <c r="F27" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="13" t="n">
         <f aca="false">E27-F27</f>
-        <v>29399.52</v>
+        <v>38598.09</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1855,24 +1855,24 @@
         <v>23</v>
       </c>
       <c r="B28" s="11" t="n">
-        <v>139620.5</v>
+        <v>178275.5</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>68507.38</v>
+        <v>80340.19</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>41320.31</v>
+        <v>55677.5</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">B28-C28-D28</f>
-        <v>29792.81</v>
+        <v>42257.81</v>
       </c>
       <c r="F28" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="13" t="n">
         <f aca="false">E28-F28</f>
-        <v>29792.81</v>
+        <v>42257.81</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1880,24 +1880,24 @@
         <v>24</v>
       </c>
       <c r="B29" s="11" t="n">
-        <v>142014.5</v>
+        <v>182766.5</v>
       </c>
       <c r="C29" s="11" t="n">
-        <v>69283.61</v>
+        <v>81752.92</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>41823.04</v>
+        <v>56777.79</v>
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">B29-C29-D29</f>
-        <v>30907.85</v>
+        <v>44235.79</v>
       </c>
       <c r="F29" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">E29-F29</f>
-        <v>30907.85</v>
+        <v>44235.79</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1906,19 +1906,19 @@
       </c>
       <c r="B30" s="13" t="n">
         <f aca="false">SUM(B5:B29)</f>
-        <v>1942515.5</v>
+        <v>2233383.5</v>
       </c>
       <c r="C30" s="13" t="n">
         <f aca="false">SUM(C5:C29)</f>
-        <v>930574.51</v>
+        <v>1023471.56</v>
       </c>
       <c r="D30" s="13" t="n">
         <f aca="false">SUM(D5:D29)</f>
-        <v>691152.2</v>
+        <v>828210.44</v>
       </c>
       <c r="E30" s="13" t="n">
         <f aca="false">SUM(E5:E29)</f>
-        <v>320788.79</v>
+        <v>381701.5</v>
       </c>
       <c r="F30" s="13" t="n">
         <f aca="false">SUM(F5:F29)</f>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="G30" s="13" t="n">
         <f aca="false">SUM(G5:G29)</f>
-        <v>218788.79</v>
+        <v>279701.5</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2043,11 +2043,11 @@
       </c>
       <c r="B6" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B6</f>
-        <v>4788</v>
+        <v>5988</v>
       </c>
       <c r="C6" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C6</f>
-        <v>1197.9</v>
+        <v>1479.9</v>
       </c>
       <c r="D6" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D6</f>
@@ -2059,11 +2059,11 @@
       </c>
       <c r="F6" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G6</f>
-        <v>-8409.9</v>
+        <v>-7491.9</v>
       </c>
       <c r="G6" s="13" t="n">
         <f aca="false">G5+F6</f>
-        <v>-110409.9</v>
+        <v>-109491.9</v>
       </c>
       <c r="H6" s="16" t="str">
         <f aca="false">IF(G6&gt;=0,"Sim","Não")</f>
@@ -2076,11 +2076,11 @@
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B7</f>
-        <v>7182</v>
+        <v>8982</v>
       </c>
       <c r="C7" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C7</f>
-        <v>1796.85</v>
+        <v>2219.85</v>
       </c>
       <c r="D7" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D7</f>
@@ -2092,11 +2092,11 @@
       </c>
       <c r="F7" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G7</f>
-        <v>-6614.85</v>
+        <v>-5237.85</v>
       </c>
       <c r="G7" s="13" t="n">
         <f aca="false">G6+F7</f>
-        <v>-117024.75</v>
+        <v>-114729.75</v>
       </c>
       <c r="H7" s="16" t="str">
         <f aca="false">IF(G7&gt;=0,"Sim","Não")</f>
@@ -2109,11 +2109,11 @@
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B8</f>
-        <v>10773</v>
+        <v>13473</v>
       </c>
       <c r="C8" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C8</f>
-        <v>2695.28</v>
+        <v>3329.78</v>
       </c>
       <c r="D8" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D8</f>
@@ -2125,11 +2125,11 @@
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G8</f>
-        <v>-3922.28</v>
+        <v>-1856.78</v>
       </c>
       <c r="G8" s="13" t="n">
         <f aca="false">G7+F8</f>
-        <v>-120947.03</v>
+        <v>-116586.53</v>
       </c>
       <c r="H8" s="16" t="str">
         <f aca="false">IF(G8&gt;=0,"Sim","Não")</f>
@@ -2142,15 +2142,15 @@
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B9</f>
-        <v>23164</v>
+        <v>24967</v>
       </c>
       <c r="C9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C9</f>
-        <v>9642.5</v>
+        <v>10156.02</v>
       </c>
       <c r="D9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D9</f>
-        <v>16864.44</v>
+        <v>18116.92</v>
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F9</f>
@@ -2158,11 +2158,11 @@
       </c>
       <c r="F9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G9</f>
-        <v>-3342.94</v>
+        <v>-3305.94</v>
       </c>
       <c r="G9" s="13" t="n">
         <f aca="false">G8+F9</f>
-        <v>-124289.97</v>
+        <v>-119892.47</v>
       </c>
       <c r="H9" s="16" t="str">
         <f aca="false">IF(G9&gt;=0,"Sim","Não")</f>
@@ -2175,15 +2175,15 @@
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B10</f>
-        <v>26755</v>
+        <v>29458</v>
       </c>
       <c r="C10" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C10</f>
-        <v>10540.92</v>
+        <v>11265.95</v>
       </c>
       <c r="D10" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D10</f>
-        <v>17618.55</v>
+        <v>19217.21</v>
       </c>
       <c r="E10" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F10</f>
@@ -2191,11 +2191,11 @@
       </c>
       <c r="F10" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G10</f>
-        <v>-1404.47</v>
+        <v>-1025.16</v>
       </c>
       <c r="G10" s="13" t="n">
         <f aca="false">G9+F10</f>
-        <v>-125694.44</v>
+        <v>-120917.63</v>
       </c>
       <c r="H10" s="16" t="str">
         <f aca="false">IF(G10&gt;=0,"Sim","Não")</f>
@@ -2208,15 +2208,15 @@
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B11</f>
-        <v>34148.5</v>
+        <v>35954.5</v>
       </c>
       <c r="C11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C11</f>
-        <v>14214.59</v>
+        <v>14903.98</v>
       </c>
       <c r="D11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D11</f>
-        <v>19171.18</v>
+        <v>20808.85</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F11</f>
@@ -2224,11 +2224,11 @@
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G11</f>
-        <v>762.73</v>
+        <v>241.670000000002</v>
       </c>
       <c r="G11" s="13" t="n">
         <f aca="false">G10+F11</f>
-        <v>-124931.71</v>
+        <v>-120675.96</v>
       </c>
       <c r="H11" s="16" t="str">
         <f aca="false">IF(G11&gt;=0,"Sim","Não")</f>
@@ -2241,15 +2241,15 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B12</f>
-        <v>37739.5</v>
+        <v>40445.5</v>
       </c>
       <c r="C12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C12</f>
-        <v>15261.5</v>
+        <v>16173.83</v>
       </c>
       <c r="D12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D12</f>
-        <v>19925.29</v>
+        <v>21909.15</v>
       </c>
       <c r="E12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F12</f>
@@ -2257,11 +2257,11 @@
       </c>
       <c r="F12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G12</f>
-        <v>2552.71</v>
+        <v>2362.52</v>
       </c>
       <c r="G12" s="13" t="n">
         <f aca="false">G11+F12</f>
-        <v>-122379</v>
+        <v>-118313.44</v>
       </c>
       <c r="H12" s="16" t="str">
         <f aca="false">IF(G12&gt;=0,"Sim","Não")</f>
@@ -2274,15 +2274,15 @@
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B13</f>
-        <v>45133</v>
+        <v>46942</v>
       </c>
       <c r="C13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C13</f>
-        <v>19095.39</v>
+        <v>19881.12</v>
       </c>
       <c r="D13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D13</f>
-        <v>21477.93</v>
+        <v>23500.79</v>
       </c>
       <c r="E13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F13</f>
@@ -2290,11 +2290,11 @@
       </c>
       <c r="F13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G13</f>
-        <v>4559.68</v>
+        <v>3560.09</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">G12+F13</f>
-        <v>-117819.32</v>
+        <v>-114753.35</v>
       </c>
       <c r="H13" s="16" t="str">
         <f aca="false">IF(G13&gt;=0,"Sim","Não")</f>
@@ -2307,15 +2307,15 @@
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B14</f>
-        <v>58721</v>
+        <v>61430</v>
       </c>
       <c r="C14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C14</f>
-        <v>26572.68</v>
+        <v>27581.5</v>
       </c>
       <c r="D14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D14</f>
-        <v>24331.41</v>
+        <v>27050.35</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F14</f>
@@ -2323,11 +2323,11 @@
       </c>
       <c r="F14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G14</f>
-        <v>7816.91</v>
+        <v>6798.15</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">G13+F14</f>
-        <v>-110002.41</v>
+        <v>-107955.2</v>
       </c>
       <c r="H14" s="16" t="str">
         <f aca="false">IF(G14&gt;=0,"Sim","Não")</f>
@@ -2340,15 +2340,15 @@
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B15</f>
-        <v>56117.5</v>
+        <v>59426.5</v>
       </c>
       <c r="C15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C15</f>
-        <v>23999.25</v>
+        <v>25142.12</v>
       </c>
       <c r="D15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D15</f>
-        <v>23784.67</v>
+        <v>26559.49</v>
       </c>
       <c r="E15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F15</f>
@@ -2356,11 +2356,11 @@
       </c>
       <c r="F15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G15</f>
-        <v>8333.58</v>
+        <v>7724.89</v>
       </c>
       <c r="G15" s="13" t="n">
         <f aca="false">G14+F15</f>
-        <v>-101668.83</v>
+        <v>-100230.31</v>
       </c>
       <c r="H15" s="16" t="str">
         <f aca="false">IF(G15&gt;=0,"Sim","Não")</f>
@@ -2373,15 +2373,15 @@
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B16</f>
-        <v>69705.5</v>
+        <v>73914.5</v>
       </c>
       <c r="C16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C16</f>
-        <v>31505.24</v>
+        <v>32956.18</v>
       </c>
       <c r="D16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D16</f>
-        <v>26638.15</v>
+        <v>30109.05</v>
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F16</f>
@@ -2389,11 +2389,11 @@
       </c>
       <c r="F16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G16</f>
-        <v>11562.11</v>
+        <v>10849.27</v>
       </c>
       <c r="G16" s="13" t="n">
         <f aca="false">G15+F16</f>
-        <v>-90106.72</v>
+        <v>-89381.04</v>
       </c>
       <c r="H16" s="16" t="str">
         <f aca="false">IF(G16&gt;=0,"Sim","Não")</f>
@@ -2406,15 +2406,15 @@
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B17</f>
-        <v>62102.5</v>
+        <v>66911.5</v>
       </c>
       <c r="C17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C17</f>
-        <v>25834.25</v>
+        <v>27417.83</v>
       </c>
       <c r="D17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D17</f>
-        <v>25041.53</v>
+        <v>28393.32</v>
       </c>
       <c r="E17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F17</f>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="F17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G17</f>
-        <v>11226.72</v>
+        <v>11100.35</v>
       </c>
       <c r="G17" s="13" t="n">
         <f aca="false">G16+F17</f>
-        <v>-78880</v>
+        <v>-78280.69</v>
       </c>
       <c r="H17" s="16" t="str">
         <f aca="false">IF(G17&gt;=0,"Sim","Não")</f>
@@ -2439,15 +2439,15 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B18</f>
-        <v>100684</v>
+        <v>104896</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C18</f>
-        <v>49617.01</v>
+        <v>51415.58</v>
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D18</f>
-        <v>33143.64</v>
+        <v>37699.52</v>
       </c>
       <c r="E18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F18</f>
@@ -2455,11 +2455,11 @@
       </c>
       <c r="F18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G18</f>
-        <v>17923.35</v>
+        <v>15780.9</v>
       </c>
       <c r="G18" s="13" t="n">
         <f aca="false">G17+F18</f>
-        <v>-60956.65</v>
+        <v>-62499.79</v>
       </c>
       <c r="H18" s="16" t="str">
         <f aca="false">IF(G18&gt;=0,"Sim","Não")</f>
@@ -2472,15 +2472,15 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B19</f>
-        <v>103078</v>
+        <v>109387</v>
       </c>
       <c r="C19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C19</f>
-        <v>50678.8</v>
+        <v>53122</v>
       </c>
       <c r="D19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D19</f>
-        <v>33646.38</v>
+        <v>38799.82</v>
       </c>
       <c r="E19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F19</f>
@@ -2488,11 +2488,11 @@
       </c>
       <c r="F19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G19</f>
-        <v>18752.82</v>
+        <v>17465.18</v>
       </c>
       <c r="G19" s="13" t="n">
         <f aca="false">G18+F19</f>
-        <v>-42203.83</v>
+        <v>-45034.61</v>
       </c>
       <c r="H19" s="16" t="str">
         <f aca="false">IF(G19&gt;=0,"Sim","Não")</f>
@@ -2505,15 +2505,15 @@
       </c>
       <c r="B20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B20</f>
-        <v>110471.5</v>
+        <v>120374.5</v>
       </c>
       <c r="C20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C20</f>
-        <v>54824.4</v>
+        <v>58240.6</v>
       </c>
       <c r="D20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D20</f>
-        <v>35199.01</v>
+        <v>41491.75</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F20</f>
@@ -2521,11 +2521,11 @@
       </c>
       <c r="F20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G20</f>
-        <v>20448.09</v>
+        <v>20642.15</v>
       </c>
       <c r="G20" s="13" t="n">
         <f aca="false">G19+F20</f>
-        <v>-21755.74</v>
+        <v>-24392.46</v>
       </c>
       <c r="H20" s="16" t="str">
         <f aca="false">IF(G20&gt;=0,"Sim","Não")</f>
@@ -2538,15 +2538,15 @@
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B21</f>
-        <v>112865.5</v>
+        <v>126362.5</v>
       </c>
       <c r="C21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C21</f>
-        <v>55737.18</v>
+        <v>60218.42</v>
       </c>
       <c r="D21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D21</f>
-        <v>35701.75</v>
+        <v>42958.81</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F21</f>
@@ -2554,11 +2554,11 @@
       </c>
       <c r="F21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G21</f>
-        <v>21426.57</v>
+        <v>23185.27</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">G20+F21</f>
-        <v>-329.170000000006</v>
+        <v>-1207.19</v>
       </c>
       <c r="H21" s="16" t="str">
         <f aca="false">IF(G21&gt;=0,"Sim","Não")</f>
@@ -2571,15 +2571,15 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B22</f>
-        <v>120259</v>
+        <v>135853</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C22</f>
-        <v>59916.83</v>
+        <v>65015.49</v>
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D22</f>
-        <v>37254.39</v>
+        <v>45283.99</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F22</f>
@@ -2587,11 +2587,11 @@
       </c>
       <c r="F22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G22</f>
-        <v>23087.78</v>
+        <v>25553.52</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">G21+F22</f>
-        <v>22758.61</v>
+        <v>24346.33</v>
       </c>
       <c r="H22" s="16" t="str">
         <f aca="false">IF(G22&gt;=0,"Sim","Não")</f>
@@ -2604,15 +2604,15 @@
       </c>
       <c r="B23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B23</f>
-        <v>122653</v>
+        <v>141841</v>
       </c>
       <c r="C23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C23</f>
-        <v>60848.72</v>
+        <v>66978.03</v>
       </c>
       <c r="D23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D23</f>
-        <v>37757.13</v>
+        <v>46751.05</v>
       </c>
       <c r="E23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F23</f>
@@ -2620,11 +2620,11 @@
       </c>
       <c r="F23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G23</f>
-        <v>24047.15</v>
+        <v>28111.92</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">G22+F23</f>
-        <v>46805.76</v>
+        <v>52458.25</v>
       </c>
       <c r="H23" s="16" t="str">
         <f aca="false">IF(G23&gt;=0,"Sim","Não")</f>
@@ -2637,15 +2637,15 @@
       </c>
       <c r="B24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B24</f>
-        <v>135044</v>
+        <v>157826</v>
       </c>
       <c r="C24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C24</f>
-        <v>68407.36</v>
+        <v>75702.62</v>
       </c>
       <c r="D24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D24</f>
-        <v>40359.24</v>
+        <v>50667.37</v>
       </c>
       <c r="E24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F24</f>
@@ -2653,11 +2653,11 @@
       </c>
       <c r="F24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G24</f>
-        <v>26277.4</v>
+        <v>31456.01</v>
       </c>
       <c r="G24" s="13" t="n">
         <f aca="false">G23+F24</f>
-        <v>73083.16</v>
+        <v>83914.26</v>
       </c>
       <c r="H24" s="16" t="str">
         <f aca="false">IF(G24&gt;=0,"Sim","Não")</f>
@@ -2670,15 +2670,15 @@
       </c>
       <c r="B25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B25</f>
-        <v>137438</v>
+        <v>163814</v>
       </c>
       <c r="C25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C25</f>
-        <v>69293.65</v>
+        <v>77638.6</v>
       </c>
       <c r="D25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D25</f>
-        <v>40861.98</v>
+        <v>52134.43</v>
       </c>
       <c r="E25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F25</f>
@@ -2686,11 +2686,11 @@
       </c>
       <c r="F25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G25</f>
-        <v>27282.37</v>
+        <v>34040.97</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">G24+F25</f>
-        <v>100365.53</v>
+        <v>117955.23</v>
       </c>
       <c r="H25" s="16" t="str">
         <f aca="false">IF(G25&gt;=0,"Sim","Não")</f>
@@ -2703,15 +2703,15 @@
       </c>
       <c r="B26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B26</f>
-        <v>139832</v>
+        <v>169802</v>
       </c>
       <c r="C26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C26</f>
-        <v>70144.2</v>
+        <v>79545.93</v>
       </c>
       <c r="D26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D26</f>
-        <v>41364.72</v>
+        <v>53601.49</v>
       </c>
       <c r="E26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F26</f>
@@ -2719,11 +2719,11 @@
       </c>
       <c r="F26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G26</f>
-        <v>28323.08</v>
+        <v>36654.58</v>
       </c>
       <c r="G26" s="13" t="n">
         <f aca="false">G25+F26</f>
-        <v>128688.61</v>
+        <v>154609.81</v>
       </c>
       <c r="H26" s="16" t="str">
         <f aca="false">IF(G26&gt;=0,"Sim","Não")</f>
@@ -2736,15 +2736,15 @@
       </c>
       <c r="B27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B27</f>
-        <v>142226</v>
+        <v>174293</v>
       </c>
       <c r="C27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C27</f>
-        <v>70959.02</v>
+        <v>80993.12</v>
       </c>
       <c r="D27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D27</f>
-        <v>41867.46</v>
+        <v>54701.79</v>
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F27</f>
@@ -2752,11 +2752,11 @@
       </c>
       <c r="F27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G27</f>
-        <v>29399.52</v>
+        <v>38598.09</v>
       </c>
       <c r="G27" s="13" t="n">
         <f aca="false">G26+F27</f>
-        <v>158088.13</v>
+        <v>193207.9</v>
       </c>
       <c r="H27" s="16" t="str">
         <f aca="false">IF(G27&gt;=0,"Sim","Não")</f>
@@ -2769,15 +2769,15 @@
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B28</f>
-        <v>139620.5</v>
+        <v>178275.5</v>
       </c>
       <c r="C28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C28</f>
-        <v>68507.38</v>
+        <v>80340.19</v>
       </c>
       <c r="D28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D28</f>
-        <v>41320.31</v>
+        <v>55677.5</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F28</f>
@@ -2785,11 +2785,11 @@
       </c>
       <c r="F28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G28</f>
-        <v>29792.81</v>
+        <v>42257.81</v>
       </c>
       <c r="G28" s="13" t="n">
         <f aca="false">G27+F28</f>
-        <v>187880.94</v>
+        <v>235465.71</v>
       </c>
       <c r="H28" s="16" t="str">
         <f aca="false">IF(G28&gt;=0,"Sim","Não")</f>
@@ -2802,15 +2802,15 @@
       </c>
       <c r="B29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B29</f>
-        <v>142014.5</v>
+        <v>182766.5</v>
       </c>
       <c r="C29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C29</f>
-        <v>69283.61</v>
+        <v>81752.92</v>
       </c>
       <c r="D29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D29</f>
-        <v>41823.04</v>
+        <v>56777.79</v>
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F29</f>
@@ -2818,11 +2818,11 @@
       </c>
       <c r="F29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G29</f>
-        <v>30907.85</v>
+        <v>44235.79</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">G28+F29</f>
-        <v>218788.79</v>
+        <v>279701.5</v>
       </c>
       <c r="H29" s="16" t="str">
         <f aca="false">IF(G29&gt;=0,"Sim","Não")</f>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="F32" s="17" t="n">
         <f aca="false">MAX(0,-MIN(G5:G29))</f>
-        <v>125694.44</v>
+        <v>120917.63</v>
       </c>
       <c r="G32" s="18" t="s">
         <v>45</v>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G6</f>
-        <v>-8409.9</v>
+        <v>-7491.9</v>
       </c>
       <c r="C12" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A12</f>
@@ -3029,11 +3029,11 @@
       </c>
       <c r="D12" s="12" t="n">
         <f aca="false">B12*C12</f>
-        <v>-8260.4877465306</v>
+        <v>-7358.79714957759</v>
       </c>
       <c r="E12" s="13" t="n">
         <f aca="false">E11+D12</f>
-        <v>-110260.487746531</v>
+        <v>-109358.797149578</v>
       </c>
       <c r="F12" s="16" t="str">
         <f aca="false">IF(E12&gt;=0,"Sim","Não")</f>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G7</f>
-        <v>-6614.85</v>
+        <v>-5237.85</v>
       </c>
       <c r="C13" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A13</f>
@@ -3054,11 +3054,11 @@
       </c>
       <c r="D13" s="12" t="n">
         <f aca="false">B13*C13</f>
-        <v>-6381.89595582955</v>
+        <v>-5053.38952995787</v>
       </c>
       <c r="E13" s="13" t="n">
         <f aca="false">E12+D13</f>
-        <v>-116642.38370236</v>
+        <v>-114412.186679535</v>
       </c>
       <c r="F13" s="16" t="str">
         <f aca="false">IF(E13&gt;=0,"Sim","Não")</f>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G8</f>
-        <v>-3922.28</v>
+        <v>-1856.78</v>
       </c>
       <c r="C14" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A14</f>
@@ -3079,11 +3079,11 @@
       </c>
       <c r="D14" s="12" t="n">
         <f aca="false">B14*C14</f>
-        <v>-3716.91964361568</v>
+        <v>-1759.56383936708</v>
       </c>
       <c r="E14" s="13" t="n">
         <f aca="false">E13+D14</f>
-        <v>-120359.303345976</v>
+        <v>-116171.750518903</v>
       </c>
       <c r="F14" s="16" t="str">
         <f aca="false">IF(E14&gt;=0,"Sim","Não")</f>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G9</f>
-        <v>-3342.94</v>
+        <v>-3305.94</v>
       </c>
       <c r="C15" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A15</f>
@@ -3104,11 +3104,11 @@
       </c>
       <c r="D15" s="12" t="n">
         <f aca="false">B15*C15</f>
-        <v>-3111.63050244808</v>
+        <v>-3077.19065949829</v>
       </c>
       <c r="E15" s="13" t="n">
         <f aca="false">E14+D15</f>
-        <v>-123470.933848424</v>
+        <v>-119248.941178401</v>
       </c>
       <c r="F15" s="16" t="str">
         <f aca="false">IF(E15&gt;=0,"Sim","Não")</f>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G10</f>
-        <v>-1404.47</v>
+        <v>-1025.16</v>
       </c>
       <c r="C16" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A16</f>
@@ -3129,11 +3129,11 @@
       </c>
       <c r="D16" s="12" t="n">
         <f aca="false">B16*C16</f>
-        <v>-1284.06427947665</v>
+        <v>-937.272662818201</v>
       </c>
       <c r="E16" s="13" t="n">
         <f aca="false">E15+D16</f>
-        <v>-124754.998127901</v>
+        <v>-120186.213841219</v>
       </c>
       <c r="F16" s="16" t="str">
         <f aca="false">IF(E16&gt;=0,"Sim","Não")</f>
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G11</f>
-        <v>762.73</v>
+        <v>241.670000000002</v>
       </c>
       <c r="C17" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A17</f>
@@ -3154,11 +3154,11 @@
       </c>
       <c r="D17" s="12" t="n">
         <f aca="false">B17*C17</f>
-        <v>684.95176007441</v>
+        <v>217.026066704055</v>
       </c>
       <c r="E17" s="13" t="n">
         <f aca="false">E16+D17</f>
-        <v>-124070.046367826</v>
+        <v>-119969.187774515</v>
       </c>
       <c r="F17" s="16" t="str">
         <f aca="false">IF(E17&gt;=0,"Sim","Não")</f>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G12</f>
-        <v>2552.71</v>
+        <v>2362.52</v>
       </c>
       <c r="C18" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A18</f>
@@ -3179,11 +3179,11 @@
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">B18*C18</f>
-        <v>2251.67391501995</v>
+        <v>2083.91264879791</v>
       </c>
       <c r="E18" s="13" t="n">
         <f aca="false">E17+D18</f>
-        <v>-121818.372452806</v>
+        <v>-117885.275125717</v>
       </c>
       <c r="F18" s="16" t="str">
         <f aca="false">IF(E18&gt;=0,"Sim","Não")</f>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G13</f>
-        <v>4559.68</v>
+        <v>3560.09</v>
       </c>
       <c r="C19" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A19</f>
@@ -3204,11 +3204,11 @@
       </c>
       <c r="D19" s="12" t="n">
         <f aca="false">B19*C19</f>
-        <v>3950.51069019917</v>
+        <v>3084.46505085251</v>
       </c>
       <c r="E19" s="13" t="n">
         <f aca="false">E18+D19</f>
-        <v>-117867.861762607</v>
+        <v>-114800.810074865</v>
       </c>
       <c r="F19" s="16" t="str">
         <f aca="false">IF(E19&gt;=0,"Sim","Não")</f>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="B20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G14</f>
-        <v>7816.91</v>
+        <v>6798.15</v>
       </c>
       <c r="C20" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A20</f>
@@ -3229,11 +3229,11 @@
       </c>
       <c r="D20" s="12" t="n">
         <f aca="false">B20*C20</f>
-        <v>6652.25437574861</v>
+        <v>5785.28127923891</v>
       </c>
       <c r="E20" s="13" t="n">
         <f aca="false">E19+D20</f>
-        <v>-111215.607386858</v>
+        <v>-109015.528795626</v>
       </c>
       <c r="F20" s="16" t="str">
         <f aca="false">IF(E20&gt;=0,"Sim","Não")</f>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G15</f>
-        <v>8333.58</v>
+        <v>7724.89</v>
       </c>
       <c r="C21" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A21</f>
@@ -3254,11 +3254,11 @@
       </c>
       <c r="D21" s="12" t="n">
         <f aca="false">B21*C21</f>
-        <v>6965.9476214782</v>
+        <v>6457.15036295095</v>
       </c>
       <c r="E21" s="13" t="n">
         <f aca="false">E20+D21</f>
-        <v>-104249.65976538</v>
+        <v>-102558.378432675</v>
       </c>
       <c r="F21" s="16" t="str">
         <f aca="false">IF(E21&gt;=0,"Sim","Não")</f>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G16</f>
-        <v>11562.11</v>
+        <v>10849.27</v>
       </c>
       <c r="C22" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A22</f>
@@ -3279,11 +3279,11 @@
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">B22*C22</f>
-        <v>9492.93598250678</v>
+        <v>8907.66698871845</v>
       </c>
       <c r="E22" s="13" t="n">
         <f aca="false">E21+D22</f>
-        <v>-94756.7237828734</v>
+        <v>-93650.7114439562</v>
       </c>
       <c r="F22" s="16" t="str">
         <f aca="false">IF(E22&gt;=0,"Sim","Não")</f>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="B23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G17</f>
-        <v>11226.72</v>
+        <v>11100.35</v>
       </c>
       <c r="C23" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A23</f>
@@ -3304,11 +3304,11 @@
       </c>
       <c r="D23" s="12" t="n">
         <f aca="false">B23*C23</f>
-        <v>9053.8064516129</v>
+        <v>8951.89516129032</v>
       </c>
       <c r="E23" s="13" t="n">
         <f aca="false">E22+D23</f>
-        <v>-85702.9173312605</v>
+        <v>-84698.8162826659</v>
       </c>
       <c r="F23" s="16" t="str">
         <f aca="false">IF(E23&gt;=0,"Sim","Não")</f>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="B24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G18</f>
-        <v>17923.35</v>
+        <v>15780.9</v>
       </c>
       <c r="C24" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A24</f>
@@ -3329,11 +3329,11 @@
       </c>
       <c r="D24" s="12" t="n">
         <f aca="false">B24*C24</f>
-        <v>14197.5157784258</v>
+        <v>12500.4297047014</v>
       </c>
       <c r="E24" s="13" t="n">
         <f aca="false">E23+D24</f>
-        <v>-71505.4015528347</v>
+        <v>-72198.3865779645</v>
       </c>
       <c r="F24" s="16" t="str">
         <f aca="false">IF(E24&gt;=0,"Sim","Não")</f>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="B25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G19</f>
-        <v>18752.82</v>
+        <v>17465.18</v>
       </c>
       <c r="C25" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A25</f>
@@ -3354,11 +3354,11 @@
       </c>
       <c r="D25" s="12" t="n">
         <f aca="false">B25*C25</f>
-        <v>14590.6493037781</v>
+        <v>13588.7997862379</v>
       </c>
       <c r="E25" s="13" t="n">
         <f aca="false">E24+D25</f>
-        <v>-56914.7522490567</v>
+        <v>-58609.5867917266</v>
       </c>
       <c r="F25" s="16" t="str">
         <f aca="false">IF(E25&gt;=0,"Sim","Não")</f>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="B26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G20</f>
-        <v>20448.09</v>
+        <v>20642.15</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A26</f>
@@ -3379,11 +3379,11 @@
       </c>
       <c r="D26" s="12" t="n">
         <f aca="false">B26*C26</f>
-        <v>15627.0010570344</v>
+        <v>15775.3071249913</v>
       </c>
       <c r="E26" s="13" t="n">
         <f aca="false">E25+D26</f>
-        <v>-41287.7511920222</v>
+        <v>-42834.2796667353</v>
       </c>
       <c r="F26" s="16" t="str">
         <f aca="false">IF(E26&gt;=0,"Sim","Não")</f>
@@ -3396,7 +3396,7 @@
       </c>
       <c r="B27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G21</f>
-        <v>21426.57</v>
+        <v>23185.27</v>
       </c>
       <c r="C27" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A27</f>
@@ -3404,11 +3404,11 @@
       </c>
       <c r="D27" s="12" t="n">
         <f aca="false">B27*C27</f>
-        <v>16083.8645543316</v>
+        <v>17404.0335123917</v>
       </c>
       <c r="E27" s="13" t="n">
         <f aca="false">E26+D27</f>
-        <v>-25203.8866376907</v>
+        <v>-25430.2461543436</v>
       </c>
       <c r="F27" s="16" t="str">
         <f aca="false">IF(E27&gt;=0,"Sim","Não")</f>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G22</f>
-        <v>23087.78</v>
+        <v>25553.52</v>
       </c>
       <c r="C28" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A28</f>
@@ -3429,11 +3429,11 @@
       </c>
       <c r="D28" s="12" t="n">
         <f aca="false">B28*C28</f>
-        <v>17022.9486122393</v>
+        <v>18840.9737888107</v>
       </c>
       <c r="E28" s="13" t="n">
         <f aca="false">E27+D28</f>
-        <v>-8180.93802545139</v>
+        <v>-6589.27236553283</v>
       </c>
       <c r="F28" s="16" t="str">
         <f aca="false">IF(E28&gt;=0,"Sim","Não")</f>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G23</f>
-        <v>24047.15</v>
+        <v>28111.92</v>
       </c>
       <c r="C29" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A29</f>
@@ -3454,11 +3454,11 @@
       </c>
       <c r="D29" s="12" t="n">
         <f aca="false">B29*C29</f>
-        <v>17415.3049944885</v>
+        <v>20359.0721054537</v>
       </c>
       <c r="E29" s="13" t="n">
         <f aca="false">E28+D29</f>
-        <v>9234.36696903715</v>
+        <v>13769.7997399209</v>
       </c>
       <c r="F29" s="16" t="str">
         <f aca="false">IF(E29&gt;=0,"Sim","Não")</f>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B30" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G24</f>
-        <v>26277.4</v>
+        <v>31456.01</v>
       </c>
       <c r="C30" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A30</f>
@@ -3479,11 +3479,11 @@
       </c>
       <c r="D30" s="12" t="n">
         <f aca="false">B30*C30</f>
-        <v>18692.3852761111</v>
+        <v>22376.1809832481</v>
       </c>
       <c r="E30" s="13" t="n">
         <f aca="false">E29+D30</f>
-        <v>27926.7522451483</v>
+        <v>36145.980723169</v>
       </c>
       <c r="F30" s="16" t="str">
         <f aca="false">IF(E30&gt;=0,"Sim","Não")</f>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="B31" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G25</f>
-        <v>27282.37</v>
+        <v>34040.97</v>
       </c>
       <c r="C31" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A31</f>
@@ -3504,11 +3504,11 @@
       </c>
       <c r="D31" s="12" t="n">
         <f aca="false">B31*C31</f>
-        <v>19062.4749450034</v>
+        <v>23784.778878397</v>
       </c>
       <c r="E31" s="13" t="n">
         <f aca="false">E30+D31</f>
-        <v>46989.2271901517</v>
+        <v>59930.759601566</v>
       </c>
       <c r="F31" s="16" t="str">
         <f aca="false">IF(E31&gt;=0,"Sim","Não")</f>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="B32" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G26</f>
-        <v>28323.08</v>
+        <v>36654.58</v>
       </c>
       <c r="C32" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A32</f>
@@ -3529,11 +3529,11 @@
       </c>
       <c r="D32" s="12" t="n">
         <f aca="false">B32*C32</f>
-        <v>19438.0426190885</v>
+        <v>25155.9254228279</v>
       </c>
       <c r="E32" s="13" t="n">
         <f aca="false">E31+D32</f>
-        <v>66427.2698092401</v>
+        <v>85086.6850243939</v>
       </c>
       <c r="F32" s="16" t="str">
         <f aca="false">IF(E32&gt;=0,"Sim","Não")</f>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="B33" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G27</f>
-        <v>29399.52</v>
+        <v>38598.09</v>
       </c>
       <c r="C33" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A33</f>
@@ -3554,11 +3554,11 @@
       </c>
       <c r="D33" s="12" t="n">
         <f aca="false">B33*C33</f>
-        <v>19818.3343208461</v>
+        <v>26019.1272431015</v>
       </c>
       <c r="E33" s="13" t="n">
         <f aca="false">E32+D33</f>
-        <v>86245.6041300863</v>
+        <v>111105.812267495</v>
       </c>
       <c r="F33" s="16" t="str">
         <f aca="false">IF(E33&gt;=0,"Sim","Não")</f>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B34" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G28</f>
-        <v>29792.81</v>
+        <v>42257.81</v>
       </c>
       <c r="C34" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A34</f>
@@ -3579,11 +3579,11 @@
       </c>
       <c r="D34" s="12" t="n">
         <f aca="false">B34*C34</f>
-        <v>19726.6453617914</v>
+        <v>27980.0673933061</v>
       </c>
       <c r="E34" s="13" t="n">
         <f aca="false">E33+D34</f>
-        <v>105972.249491878</v>
+        <v>139085.879660802</v>
       </c>
       <c r="F34" s="16" t="str">
         <f aca="false">IF(E34&gt;=0,"Sim","Não")</f>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="B35" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G29</f>
-        <v>30907.85</v>
+        <v>44235.79</v>
       </c>
       <c r="C35" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A35</f>
@@ -3604,11 +3604,11 @@
       </c>
       <c r="D35" s="12" t="n">
         <f aca="false">B35*C35</f>
-        <v>20101.3592611862</v>
+        <v>28769.3743496358</v>
       </c>
       <c r="E35" s="13" t="n">
         <f aca="false">E34+D35</f>
-        <v>126073.608753064</v>
+        <v>167855.254010437</v>
       </c>
       <c r="F35" s="16" t="str">
         <f aca="false">IF(E35&gt;=0,"Sim","Não")</f>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B38" s="24" t="n">
         <f aca="false">SUM(D11:D35)</f>
-        <v>126073.608753064</v>
+        <v>167855.254010437</v>
       </c>
       <c r="C38" s="25" t="str">
         <f aca="false">IF(B38&gt;0,"VIÁVEL: o projeto gera mais do que a taxa exigida",IF(B38&lt;0,"INVIÁVEL: o projeto rende menos que a taxa exigida","EQUILÍBRIO: rende exatamente a taxa exigida"))</f>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="B39" s="26" t="n">
         <f aca="false">IFERROR(IRR(B11:B35),"Não calculável")</f>
-        <v>0.0615783401950765</v>
+        <v>0.0704388471707102</v>
       </c>
       <c r="C39" s="25" t="str">
         <f aca="false">IF(ISNUMBER(B39),IF(B39&gt;B7,"VIÁVEL: TIR maior que a taxa de desconto","INVIÁVEL: TIR menor ou igual à taxa de desconto"),"Sem TIR: o fluxo precisa ter valores negativos E positivos")</f>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="B40" s="26" t="n">
         <f aca="false">IF(ISNUMBER(B39),IF(B6="Mensal",(1+B39)^12-1,B39),"Não calculável")</f>
-        <v>1.04844631392788</v>
+        <v>1.26330112699677</v>
       </c>
       <c r="C40" s="25" t="str">
         <f aca="false">"Compare com a taxa anual de "&amp;ROUND(B5*100,2)&amp;"%"</f>
@@ -3684,11 +3684,11 @@
       </c>
       <c r="B42" s="26" t="n">
         <f aca="false">IF(B41=0,"-",B38/B41)</f>
-        <v>1.23601577208886</v>
+        <v>1.64563974520037</v>
       </c>
       <c r="C42" s="25" t="str">
         <f aca="false">"Para cada R$ 100 de investimento inicial, o projeto gera R$ "&amp;IF(ISNUMBER(B42),ROUND(B42*100,2),"-")&amp;" de VPL acima da taxa exigida"</f>
-        <v>Para cada R$ 100 de investimento inicial, o projeto gera R$ 123.6 de VPL acima da taxa exigida</v>
+        <v>Para cada R$ 100 de investimento inicial, o projeto gera R$ 164.56 de VPL acima da taxa exigida</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="B45" s="24" t="n">
         <f aca="false">'Necessidade de Caixa e Payback'!F32</f>
-        <v>125694.44</v>
+        <v>120917.63</v>
       </c>
       <c r="C45" s="25" t="str">
         <f aca="false">"Dinheiro que os sócios precisam ter para cobrir o pior momento"</f>

</xml_diff>

<commit_message>
Book Sprint and Scale at full price in the month of sale
Payment no longer follows delivery: the client pays by Pix or card and
Precept receives the full amount when the sale closes. Scale revenue is
now Scales sold x R$ 29.997 (not 6 monthly installments), and its
variable costs (specialists, commissions, R$ 1.200 of visits) are booked
with the sale. Partner pay stays at 3.5% each; break-even stays at
month 6 with every later month positive. VPL at 24% a.a. goes to
R$ 172,5 mil, TIR 131%, payback month 16.

The form now shows quantities that multiply exactly to each revenue
line (Scale as 11 / 12 per month). Planning document, pitch slides
11/12/16 and the Matriz page drop the installment wording; the Matriz
HTML is saved here because the artifact could not be republished.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016kLWp3PkVdryYcjkVkag3m
</commit_message>
<xml_diff>
--- a/precept-financeiro/Planilha_Financeira_Precept.xlsx
+++ b/precept-financeiro/Planilha_Financeira_Precept.xlsx
@@ -1383,21 +1383,21 @@
         <v>24967</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>10156.02</v>
+        <v>10156.03</v>
       </c>
       <c r="D9" s="11" t="n">
         <v>18116.92</v>
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">B9-C9-D9</f>
-        <v>-3305.94</v>
+        <v>-3305.95</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="13" t="n">
         <f aca="false">E9-F9</f>
-        <v>-3305.94</v>
+        <v>-3305.95</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1430,24 +1430,24 @@
         <v>6</v>
       </c>
       <c r="B11" s="11" t="n">
-        <v>35954.5</v>
+        <v>60952</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>14903.98</v>
+        <v>30336.88</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>20808.85</v>
+        <v>26933.24</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">B11-C11-D11</f>
-        <v>241.670000000002</v>
+        <v>3681.88</v>
       </c>
       <c r="F11" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="13" t="n">
         <f aca="false">E11-F11</f>
-        <v>241.670000000002</v>
+        <v>3681.88</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1455,24 +1455,24 @@
         <v>7</v>
       </c>
       <c r="B12" s="11" t="n">
-        <v>40445.5</v>
+        <v>35446</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>16173.83</v>
+        <v>13185.46</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>21909.15</v>
+        <v>20684.27</v>
       </c>
       <c r="E12" s="12" t="n">
         <f aca="false">B12-C12-D12</f>
-        <v>2362.52</v>
+        <v>1576.27</v>
       </c>
       <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="13" t="n">
         <f aca="false">E12-F12</f>
-        <v>2362.52</v>
+        <v>1576.27</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1480,24 +1480,24 @@
         <v>8</v>
       </c>
       <c r="B13" s="11" t="n">
-        <v>46942</v>
+        <v>66940</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>19881.12</v>
+        <v>32473.39</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>23500.79</v>
+        <v>28400.3</v>
       </c>
       <c r="E13" s="12" t="n">
         <f aca="false">B13-C13-D13</f>
-        <v>3560.09</v>
+        <v>6066.31</v>
       </c>
       <c r="F13" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">E13-F13</f>
-        <v>3560.09</v>
+        <v>6066.31</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1505,24 +1505,24 @@
         <v>9</v>
       </c>
       <c r="B14" s="11" t="n">
-        <v>61430</v>
+        <v>51431</v>
       </c>
       <c r="C14" s="11" t="n">
-        <v>27581.5</v>
+        <v>21468.56</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>27050.35</v>
+        <v>24600.6</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">B14-C14-D14</f>
-        <v>6798.15</v>
+        <v>5361.84</v>
       </c>
       <c r="F14" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">E14-F14</f>
-        <v>6798.15</v>
+        <v>5361.84</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1530,24 +1530,24 @@
         <v>10</v>
       </c>
       <c r="B15" s="11" t="n">
-        <v>59426.5</v>
+        <v>74425</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>25142.12</v>
+        <v>34750.33</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>26559.49</v>
+        <v>30234.12</v>
       </c>
       <c r="E15" s="12" t="n">
         <f aca="false">B15-C15-D15</f>
-        <v>7724.89</v>
+        <v>9440.55</v>
       </c>
       <c r="F15" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="13" t="n">
         <f aca="false">E15-F15</f>
-        <v>7724.89</v>
+        <v>9440.55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1555,24 +1555,24 @@
         <v>11</v>
       </c>
       <c r="B16" s="11" t="n">
-        <v>73914.5</v>
+        <v>58916</v>
       </c>
       <c r="C16" s="11" t="n">
-        <v>32956.18</v>
+        <v>23690.15</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>30109.05</v>
+        <v>26434.42</v>
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">B16-C16-D16</f>
-        <v>10849.27</v>
+        <v>8791.43</v>
       </c>
       <c r="F16" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="13" t="n">
         <f aca="false">E16-F16</f>
-        <v>10849.27</v>
+        <v>8791.43</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1580,24 +1580,24 @@
         <v>12</v>
       </c>
       <c r="B17" s="11" t="n">
-        <v>66911.5</v>
+        <v>81910</v>
       </c>
       <c r="C17" s="11" t="n">
-        <v>27417.83</v>
+        <v>37031.49</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>28393.32</v>
+        <v>32067.95</v>
       </c>
       <c r="E17" s="12" t="n">
         <f aca="false">B17-C17-D17</f>
-        <v>11100.35</v>
+        <v>12810.56</v>
       </c>
       <c r="F17" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G17" s="13" t="n">
         <f aca="false">E17-F17</f>
-        <v>11100.35</v>
+        <v>12810.56</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1605,24 +1605,24 @@
         <v>13</v>
       </c>
       <c r="B18" s="11" t="n">
-        <v>104896</v>
+        <v>114895</v>
       </c>
       <c r="C18" s="11" t="n">
-        <v>51415.58</v>
+        <v>57966.67</v>
       </c>
       <c r="D18" s="11" t="n">
-        <v>37699.52</v>
+        <v>40149.28</v>
       </c>
       <c r="E18" s="12" t="n">
         <f aca="false">B18-C18-D18</f>
-        <v>15780.9</v>
+        <v>16779.05</v>
       </c>
       <c r="F18" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="13" t="n">
         <f aca="false">E18-F18</f>
-        <v>15780.9</v>
+        <v>16779.05</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1630,24 +1630,24 @@
         <v>14</v>
       </c>
       <c r="B19" s="11" t="n">
-        <v>109387</v>
+        <v>119386</v>
       </c>
       <c r="C19" s="11" t="n">
-        <v>53122</v>
+        <v>59681.17</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>38799.82</v>
+        <v>41249.57</v>
       </c>
       <c r="E19" s="12" t="n">
         <f aca="false">B19-C19-D19</f>
-        <v>17465.18</v>
+        <v>18455.26</v>
       </c>
       <c r="F19" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G19" s="13" t="n">
         <f aca="false">E19-F19</f>
-        <v>17465.18</v>
+        <v>18455.26</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1655,24 +1655,24 @@
         <v>15</v>
       </c>
       <c r="B20" s="11" t="n">
-        <v>120374.5</v>
+        <v>125374</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>58240.6</v>
+        <v>61627.13</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>41491.75</v>
+        <v>42716.63</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">B20-C20-D20</f>
-        <v>20642.15</v>
+        <v>21030.24</v>
       </c>
       <c r="F20" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="13" t="n">
         <f aca="false">E20-F20</f>
-        <v>20642.15</v>
+        <v>21030.24</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1680,24 +1680,24 @@
         <v>16</v>
       </c>
       <c r="B21" s="11" t="n">
-        <v>126362.5</v>
+        <v>131362</v>
       </c>
       <c r="C21" s="11" t="n">
-        <v>60218.42</v>
+        <v>63673.28</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>42958.81</v>
+        <v>44183.69</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">B21-C21-D21</f>
-        <v>23185.27</v>
+        <v>23505.03</v>
       </c>
       <c r="F21" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">E21-F21</f>
-        <v>23185.27</v>
+        <v>23505.03</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1708,21 +1708,21 @@
         <v>135853</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>65015.49</v>
+        <v>65224.84</v>
       </c>
       <c r="D22" s="11" t="n">
         <v>45283.99</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">B22-C22-D22</f>
-        <v>25553.52</v>
+        <v>25344.17</v>
       </c>
       <c r="F22" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">E22-F22</f>
-        <v>25553.52</v>
+        <v>25344.17</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1733,21 +1733,21 @@
         <v>141841</v>
       </c>
       <c r="C23" s="11" t="n">
-        <v>66978.03</v>
+        <v>67153.3</v>
       </c>
       <c r="D23" s="11" t="n">
         <v>46751.05</v>
       </c>
       <c r="E23" s="12" t="n">
         <f aca="false">B23-C23-D23</f>
-        <v>28111.92</v>
+        <v>27936.65</v>
       </c>
       <c r="F23" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">E23-F23</f>
-        <v>28111.92</v>
+        <v>27936.65</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1758,21 +1758,21 @@
         <v>157826</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>75702.62</v>
+        <v>75811.64</v>
       </c>
       <c r="D24" s="11" t="n">
         <v>50667.37</v>
       </c>
       <c r="E24" s="12" t="n">
         <f aca="false">B24-C24-D24</f>
-        <v>31456.01</v>
+        <v>31346.99</v>
       </c>
       <c r="F24" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="13" t="n">
         <f aca="false">E24-F24</f>
-        <v>31456.01</v>
+        <v>31346.99</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1783,21 +1783,21 @@
         <v>163814</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>77638.6</v>
+        <v>77740.04</v>
       </c>
       <c r="D25" s="11" t="n">
         <v>52134.43</v>
       </c>
       <c r="E25" s="12" t="n">
         <f aca="false">B25-C25-D25</f>
-        <v>34040.97</v>
+        <v>33939.53</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">E25-F25</f>
-        <v>34040.97</v>
+        <v>33939.53</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1808,21 +1808,21 @@
         <v>169802</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>79545.93</v>
+        <v>79602.57</v>
       </c>
       <c r="D26" s="11" t="n">
         <v>53601.49</v>
       </c>
       <c r="E26" s="12" t="n">
         <f aca="false">B26-C26-D26</f>
-        <v>36654.58</v>
+        <v>36597.94</v>
       </c>
       <c r="F26" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="13" t="n">
         <f aca="false">E26-F26</f>
-        <v>36654.58</v>
+        <v>36597.94</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1833,21 +1833,21 @@
         <v>174293</v>
       </c>
       <c r="C27" s="11" t="n">
-        <v>80993.12</v>
+        <v>81056.66</v>
       </c>
       <c r="D27" s="11" t="n">
         <v>54701.79</v>
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">B27-C27-D27</f>
-        <v>38598.09</v>
+        <v>38534.55</v>
       </c>
       <c r="F27" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="13" t="n">
         <f aca="false">E27-F27</f>
-        <v>38598.09</v>
+        <v>38534.55</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1855,24 +1855,24 @@
         <v>23</v>
       </c>
       <c r="B28" s="11" t="n">
-        <v>178275.5</v>
+        <v>153278</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>80340.19</v>
+        <v>64025.68</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>55677.5</v>
+        <v>49553.11</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">B28-C28-D28</f>
-        <v>42257.81</v>
+        <v>39699.21</v>
       </c>
       <c r="F28" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="13" t="n">
         <f aca="false">E28-F28</f>
-        <v>42257.81</v>
+        <v>39699.21</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1880,24 +1880,24 @@
         <v>24</v>
       </c>
       <c r="B29" s="11" t="n">
-        <v>182766.5</v>
+        <v>187766</v>
       </c>
       <c r="C29" s="11" t="n">
-        <v>81752.92</v>
+        <v>85049.09</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>56777.79</v>
+        <v>58002.67</v>
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">B29-C29-D29</f>
-        <v>44235.79</v>
+        <v>44714.24</v>
       </c>
       <c r="F29" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">E29-F29</f>
-        <v>44235.79</v>
+        <v>44714.24</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1906,19 +1906,19 @@
       </c>
       <c r="B30" s="13" t="n">
         <f aca="false">SUM(B5:B29)</f>
-        <v>2233383.5</v>
+        <v>2288378</v>
       </c>
       <c r="C30" s="13" t="n">
         <f aca="false">SUM(C5:C29)</f>
-        <v>1023471.56</v>
+        <v>1059999.84</v>
       </c>
       <c r="D30" s="13" t="n">
         <f aca="false">SUM(D5:D29)</f>
-        <v>828210.44</v>
+        <v>841684.1</v>
       </c>
       <c r="E30" s="13" t="n">
         <f aca="false">SUM(E5:E29)</f>
-        <v>381701.5</v>
+        <v>386694.06</v>
       </c>
       <c r="F30" s="13" t="n">
         <f aca="false">SUM(F5:F29)</f>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="G30" s="13" t="n">
         <f aca="false">SUM(G5:G29)</f>
-        <v>279701.5</v>
+        <v>284694.06</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="C9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C9</f>
-        <v>10156.02</v>
+        <v>10156.03</v>
       </c>
       <c r="D9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D9</f>
@@ -2158,11 +2158,11 @@
       </c>
       <c r="F9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G9</f>
-        <v>-3305.94</v>
+        <v>-3305.95</v>
       </c>
       <c r="G9" s="13" t="n">
         <f aca="false">G8+F9</f>
-        <v>-119892.47</v>
+        <v>-119892.48</v>
       </c>
       <c r="H9" s="16" t="str">
         <f aca="false">IF(G9&gt;=0,"Sim","Não")</f>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="G10" s="13" t="n">
         <f aca="false">G9+F10</f>
-        <v>-120917.63</v>
+        <v>-120917.64</v>
       </c>
       <c r="H10" s="16" t="str">
         <f aca="false">IF(G10&gt;=0,"Sim","Não")</f>
@@ -2208,15 +2208,15 @@
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B11</f>
-        <v>35954.5</v>
+        <v>60952</v>
       </c>
       <c r="C11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C11</f>
-        <v>14903.98</v>
+        <v>30336.88</v>
       </c>
       <c r="D11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D11</f>
-        <v>20808.85</v>
+        <v>26933.24</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F11</f>
@@ -2224,11 +2224,11 @@
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G11</f>
-        <v>241.670000000002</v>
+        <v>3681.88</v>
       </c>
       <c r="G11" s="13" t="n">
         <f aca="false">G10+F11</f>
-        <v>-120675.96</v>
+        <v>-117235.76</v>
       </c>
       <c r="H11" s="16" t="str">
         <f aca="false">IF(G11&gt;=0,"Sim","Não")</f>
@@ -2241,15 +2241,15 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B12</f>
-        <v>40445.5</v>
+        <v>35446</v>
       </c>
       <c r="C12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C12</f>
-        <v>16173.83</v>
+        <v>13185.46</v>
       </c>
       <c r="D12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D12</f>
-        <v>21909.15</v>
+        <v>20684.27</v>
       </c>
       <c r="E12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F12</f>
@@ -2257,11 +2257,11 @@
       </c>
       <c r="F12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G12</f>
-        <v>2362.52</v>
+        <v>1576.27</v>
       </c>
       <c r="G12" s="13" t="n">
         <f aca="false">G11+F12</f>
-        <v>-118313.44</v>
+        <v>-115659.49</v>
       </c>
       <c r="H12" s="16" t="str">
         <f aca="false">IF(G12&gt;=0,"Sim","Não")</f>
@@ -2274,15 +2274,15 @@
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B13</f>
-        <v>46942</v>
+        <v>66940</v>
       </c>
       <c r="C13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C13</f>
-        <v>19881.12</v>
+        <v>32473.39</v>
       </c>
       <c r="D13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D13</f>
-        <v>23500.79</v>
+        <v>28400.3</v>
       </c>
       <c r="E13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F13</f>
@@ -2290,11 +2290,11 @@
       </c>
       <c r="F13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G13</f>
-        <v>3560.09</v>
+        <v>6066.31</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">G12+F13</f>
-        <v>-114753.35</v>
+        <v>-109593.18</v>
       </c>
       <c r="H13" s="16" t="str">
         <f aca="false">IF(G13&gt;=0,"Sim","Não")</f>
@@ -2307,15 +2307,15 @@
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B14</f>
-        <v>61430</v>
+        <v>51431</v>
       </c>
       <c r="C14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C14</f>
-        <v>27581.5</v>
+        <v>21468.56</v>
       </c>
       <c r="D14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D14</f>
-        <v>27050.35</v>
+        <v>24600.6</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F14</f>
@@ -2323,11 +2323,11 @@
       </c>
       <c r="F14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G14</f>
-        <v>6798.15</v>
+        <v>5361.84</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">G13+F14</f>
-        <v>-107955.2</v>
+        <v>-104231.34</v>
       </c>
       <c r="H14" s="16" t="str">
         <f aca="false">IF(G14&gt;=0,"Sim","Não")</f>
@@ -2340,15 +2340,15 @@
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B15</f>
-        <v>59426.5</v>
+        <v>74425</v>
       </c>
       <c r="C15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C15</f>
-        <v>25142.12</v>
+        <v>34750.33</v>
       </c>
       <c r="D15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D15</f>
-        <v>26559.49</v>
+        <v>30234.12</v>
       </c>
       <c r="E15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F15</f>
@@ -2356,11 +2356,11 @@
       </c>
       <c r="F15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G15</f>
-        <v>7724.89</v>
+        <v>9440.55</v>
       </c>
       <c r="G15" s="13" t="n">
         <f aca="false">G14+F15</f>
-        <v>-100230.31</v>
+        <v>-94790.79</v>
       </c>
       <c r="H15" s="16" t="str">
         <f aca="false">IF(G15&gt;=0,"Sim","Não")</f>
@@ -2373,15 +2373,15 @@
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B16</f>
-        <v>73914.5</v>
+        <v>58916</v>
       </c>
       <c r="C16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C16</f>
-        <v>32956.18</v>
+        <v>23690.15</v>
       </c>
       <c r="D16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D16</f>
-        <v>30109.05</v>
+        <v>26434.42</v>
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F16</f>
@@ -2389,11 +2389,11 @@
       </c>
       <c r="F16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G16</f>
-        <v>10849.27</v>
+        <v>8791.43</v>
       </c>
       <c r="G16" s="13" t="n">
         <f aca="false">G15+F16</f>
-        <v>-89381.04</v>
+        <v>-85999.36</v>
       </c>
       <c r="H16" s="16" t="str">
         <f aca="false">IF(G16&gt;=0,"Sim","Não")</f>
@@ -2406,15 +2406,15 @@
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B17</f>
-        <v>66911.5</v>
+        <v>81910</v>
       </c>
       <c r="C17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C17</f>
-        <v>27417.83</v>
+        <v>37031.49</v>
       </c>
       <c r="D17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D17</f>
-        <v>28393.32</v>
+        <v>32067.95</v>
       </c>
       <c r="E17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F17</f>
@@ -2422,11 +2422,11 @@
       </c>
       <c r="F17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G17</f>
-        <v>11100.35</v>
+        <v>12810.56</v>
       </c>
       <c r="G17" s="13" t="n">
         <f aca="false">G16+F17</f>
-        <v>-78280.69</v>
+        <v>-73188.8</v>
       </c>
       <c r="H17" s="16" t="str">
         <f aca="false">IF(G17&gt;=0,"Sim","Não")</f>
@@ -2439,15 +2439,15 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B18</f>
-        <v>104896</v>
+        <v>114895</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C18</f>
-        <v>51415.58</v>
+        <v>57966.67</v>
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D18</f>
-        <v>37699.52</v>
+        <v>40149.28</v>
       </c>
       <c r="E18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F18</f>
@@ -2455,11 +2455,11 @@
       </c>
       <c r="F18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G18</f>
-        <v>15780.9</v>
+        <v>16779.05</v>
       </c>
       <c r="G18" s="13" t="n">
         <f aca="false">G17+F18</f>
-        <v>-62499.79</v>
+        <v>-56409.75</v>
       </c>
       <c r="H18" s="16" t="str">
         <f aca="false">IF(G18&gt;=0,"Sim","Não")</f>
@@ -2472,15 +2472,15 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B19</f>
-        <v>109387</v>
+        <v>119386</v>
       </c>
       <c r="C19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C19</f>
-        <v>53122</v>
+        <v>59681.17</v>
       </c>
       <c r="D19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D19</f>
-        <v>38799.82</v>
+        <v>41249.57</v>
       </c>
       <c r="E19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F19</f>
@@ -2488,11 +2488,11 @@
       </c>
       <c r="F19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G19</f>
-        <v>17465.18</v>
+        <v>18455.26</v>
       </c>
       <c r="G19" s="13" t="n">
         <f aca="false">G18+F19</f>
-        <v>-45034.61</v>
+        <v>-37954.49</v>
       </c>
       <c r="H19" s="16" t="str">
         <f aca="false">IF(G19&gt;=0,"Sim","Não")</f>
@@ -2505,15 +2505,15 @@
       </c>
       <c r="B20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B20</f>
-        <v>120374.5</v>
+        <v>125374</v>
       </c>
       <c r="C20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C20</f>
-        <v>58240.6</v>
+        <v>61627.13</v>
       </c>
       <c r="D20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D20</f>
-        <v>41491.75</v>
+        <v>42716.63</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F20</f>
@@ -2521,11 +2521,11 @@
       </c>
       <c r="F20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G20</f>
-        <v>20642.15</v>
+        <v>21030.24</v>
       </c>
       <c r="G20" s="13" t="n">
         <f aca="false">G19+F20</f>
-        <v>-24392.46</v>
+        <v>-16924.25</v>
       </c>
       <c r="H20" s="16" t="str">
         <f aca="false">IF(G20&gt;=0,"Sim","Não")</f>
@@ -2538,15 +2538,15 @@
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B21</f>
-        <v>126362.5</v>
+        <v>131362</v>
       </c>
       <c r="C21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C21</f>
-        <v>60218.42</v>
+        <v>63673.28</v>
       </c>
       <c r="D21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D21</f>
-        <v>42958.81</v>
+        <v>44183.69</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F21</f>
@@ -2554,15 +2554,15 @@
       </c>
       <c r="F21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G21</f>
-        <v>23185.27</v>
+        <v>23505.03</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">G20+F21</f>
-        <v>-1207.19</v>
+        <v>6580.77999999999</v>
       </c>
       <c r="H21" s="16" t="str">
         <f aca="false">IF(G21&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C22</f>
-        <v>65015.49</v>
+        <v>65224.84</v>
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D22</f>
@@ -2587,11 +2587,11 @@
       </c>
       <c r="F22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G22</f>
-        <v>25553.52</v>
+        <v>25344.17</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">G21+F22</f>
-        <v>24346.33</v>
+        <v>31924.95</v>
       </c>
       <c r="H22" s="16" t="str">
         <f aca="false">IF(G22&gt;=0,"Sim","Não")</f>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C23</f>
-        <v>66978.03</v>
+        <v>67153.3</v>
       </c>
       <c r="D23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D23</f>
@@ -2620,11 +2620,11 @@
       </c>
       <c r="F23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G23</f>
-        <v>28111.92</v>
+        <v>27936.65</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">G22+F23</f>
-        <v>52458.25</v>
+        <v>59861.6</v>
       </c>
       <c r="H23" s="16" t="str">
         <f aca="false">IF(G23&gt;=0,"Sim","Não")</f>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="C24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C24</f>
-        <v>75702.62</v>
+        <v>75811.64</v>
       </c>
       <c r="D24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D24</f>
@@ -2653,11 +2653,11 @@
       </c>
       <c r="F24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G24</f>
-        <v>31456.01</v>
+        <v>31346.99</v>
       </c>
       <c r="G24" s="13" t="n">
         <f aca="false">G23+F24</f>
-        <v>83914.26</v>
+        <v>91208.59</v>
       </c>
       <c r="H24" s="16" t="str">
         <f aca="false">IF(G24&gt;=0,"Sim","Não")</f>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="C25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C25</f>
-        <v>77638.6</v>
+        <v>77740.04</v>
       </c>
       <c r="D25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D25</f>
@@ -2686,11 +2686,11 @@
       </c>
       <c r="F25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G25</f>
-        <v>34040.97</v>
+        <v>33939.53</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">G24+F25</f>
-        <v>117955.23</v>
+        <v>125148.12</v>
       </c>
       <c r="H25" s="16" t="str">
         <f aca="false">IF(G25&gt;=0,"Sim","Não")</f>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="C26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C26</f>
-        <v>79545.93</v>
+        <v>79602.57</v>
       </c>
       <c r="D26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D26</f>
@@ -2719,11 +2719,11 @@
       </c>
       <c r="F26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G26</f>
-        <v>36654.58</v>
+        <v>36597.94</v>
       </c>
       <c r="G26" s="13" t="n">
         <f aca="false">G25+F26</f>
-        <v>154609.81</v>
+        <v>161746.06</v>
       </c>
       <c r="H26" s="16" t="str">
         <f aca="false">IF(G26&gt;=0,"Sim","Não")</f>
@@ -2740,7 +2740,7 @@
       </c>
       <c r="C27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C27</f>
-        <v>80993.12</v>
+        <v>81056.66</v>
       </c>
       <c r="D27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D27</f>
@@ -2752,11 +2752,11 @@
       </c>
       <c r="F27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G27</f>
-        <v>38598.09</v>
+        <v>38534.55</v>
       </c>
       <c r="G27" s="13" t="n">
         <f aca="false">G26+F27</f>
-        <v>193207.9</v>
+        <v>200280.61</v>
       </c>
       <c r="H27" s="16" t="str">
         <f aca="false">IF(G27&gt;=0,"Sim","Não")</f>
@@ -2769,15 +2769,15 @@
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B28</f>
-        <v>178275.5</v>
+        <v>153278</v>
       </c>
       <c r="C28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C28</f>
-        <v>80340.19</v>
+        <v>64025.68</v>
       </c>
       <c r="D28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D28</f>
-        <v>55677.5</v>
+        <v>49553.11</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F28</f>
@@ -2785,11 +2785,11 @@
       </c>
       <c r="F28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G28</f>
-        <v>42257.81</v>
+        <v>39699.21</v>
       </c>
       <c r="G28" s="13" t="n">
         <f aca="false">G27+F28</f>
-        <v>235465.71</v>
+        <v>239979.82</v>
       </c>
       <c r="H28" s="16" t="str">
         <f aca="false">IF(G28&gt;=0,"Sim","Não")</f>
@@ -2802,15 +2802,15 @@
       </c>
       <c r="B29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B29</f>
-        <v>182766.5</v>
+        <v>187766</v>
       </c>
       <c r="C29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C29</f>
-        <v>81752.92</v>
+        <v>85049.09</v>
       </c>
       <c r="D29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D29</f>
-        <v>56777.79</v>
+        <v>58002.67</v>
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F29</f>
@@ -2818,11 +2818,11 @@
       </c>
       <c r="F29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G29</f>
-        <v>44235.79</v>
+        <v>44714.24</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">G28+F29</f>
-        <v>279701.5</v>
+        <v>284694.06</v>
       </c>
       <c r="H29" s="16" t="str">
         <f aca="false">IF(G29&gt;=0,"Sim","Não")</f>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="F32" s="17" t="n">
         <f aca="false">MAX(0,-MIN(G5:G29))</f>
-        <v>120917.63</v>
+        <v>120917.64</v>
       </c>
       <c r="G32" s="18" t="s">
         <v>45</v>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="F33" s="19" t="n">
         <f aca="false">IFERROR(INDEX(A5:A29,MATCH("Sim",H5:H29,0)),"Não recupera")</f>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G33" s="18" t="s">
         <v>47</v>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G9</f>
-        <v>-3305.94</v>
+        <v>-3305.95</v>
       </c>
       <c r="C15" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A15</f>
@@ -3104,11 +3104,11 @@
       </c>
       <c r="D15" s="12" t="n">
         <f aca="false">B15*C15</f>
-        <v>-3077.19065949829</v>
+        <v>-3077.19996756395</v>
       </c>
       <c r="E15" s="13" t="n">
         <f aca="false">E14+D15</f>
-        <v>-119248.941178401</v>
+        <v>-119248.950486466</v>
       </c>
       <c r="F15" s="16" t="str">
         <f aca="false">IF(E15&gt;=0,"Sim","Não")</f>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="E16" s="13" t="n">
         <f aca="false">E15+D16</f>
-        <v>-120186.213841219</v>
+        <v>-120186.223149285</v>
       </c>
       <c r="F16" s="16" t="str">
         <f aca="false">IF(E16&gt;=0,"Sim","Não")</f>
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G11</f>
-        <v>241.670000000002</v>
+        <v>3681.88</v>
       </c>
       <c r="C17" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A17</f>
@@ -3154,11 +3154,11 @@
       </c>
       <c r="D17" s="12" t="n">
         <f aca="false">B17*C17</f>
-        <v>217.026066704055</v>
+        <v>3306.42584713171</v>
       </c>
       <c r="E17" s="13" t="n">
         <f aca="false">E16+D17</f>
-        <v>-119969.187774515</v>
+        <v>-116879.797302153</v>
       </c>
       <c r="F17" s="16" t="str">
         <f aca="false">IF(E17&gt;=0,"Sim","Não")</f>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G12</f>
-        <v>2362.52</v>
+        <v>1576.27</v>
       </c>
       <c r="C18" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A18</f>
@@ -3179,11 +3179,11 @@
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">B18*C18</f>
-        <v>2083.91264879791</v>
+        <v>1390.38356962933</v>
       </c>
       <c r="E18" s="13" t="n">
         <f aca="false">E17+D18</f>
-        <v>-117885.275125717</v>
+        <v>-115489.413732524</v>
       </c>
       <c r="F18" s="16" t="str">
         <f aca="false">IF(E18&gt;=0,"Sim","Não")</f>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G13</f>
-        <v>3560.09</v>
+        <v>6066.31</v>
       </c>
       <c r="C19" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A19</f>
@@ -3204,11 +3204,11 @@
       </c>
       <c r="D19" s="12" t="n">
         <f aca="false">B19*C19</f>
-        <v>3084.46505085251</v>
+        <v>5255.85622347667</v>
       </c>
       <c r="E19" s="13" t="n">
         <f aca="false">E18+D19</f>
-        <v>-114800.810074865</v>
+        <v>-110233.557509047</v>
       </c>
       <c r="F19" s="16" t="str">
         <f aca="false">IF(E19&gt;=0,"Sim","Não")</f>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="B20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G14</f>
-        <v>6798.15</v>
+        <v>5361.84</v>
       </c>
       <c r="C20" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A20</f>
@@ -3229,11 +3229,11 @@
       </c>
       <c r="D20" s="12" t="n">
         <f aca="false">B20*C20</f>
-        <v>5785.28127923891</v>
+        <v>4562.96971591894</v>
       </c>
       <c r="E20" s="13" t="n">
         <f aca="false">E19+D20</f>
-        <v>-109015.528795626</v>
+        <v>-105670.587793128</v>
       </c>
       <c r="F20" s="16" t="str">
         <f aca="false">IF(E20&gt;=0,"Sim","Não")</f>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G15</f>
-        <v>7724.89</v>
+        <v>9440.55</v>
       </c>
       <c r="C21" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A21</f>
@@ -3254,11 +3254,11 @@
       </c>
       <c r="D21" s="12" t="n">
         <f aca="false">B21*C21</f>
-        <v>6457.15036295095</v>
+        <v>7891.25163710507</v>
       </c>
       <c r="E21" s="13" t="n">
         <f aca="false">E20+D21</f>
-        <v>-102558.378432675</v>
+        <v>-97779.336156023</v>
       </c>
       <c r="F21" s="16" t="str">
         <f aca="false">IF(E21&gt;=0,"Sim","Não")</f>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G16</f>
-        <v>10849.27</v>
+        <v>8791.43</v>
       </c>
       <c r="C22" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A22</f>
@@ -3279,11 +3279,11 @@
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">B22*C22</f>
-        <v>8907.66698871845</v>
+        <v>7218.10138328468</v>
       </c>
       <c r="E22" s="13" t="n">
         <f aca="false">E21+D22</f>
-        <v>-93650.7114439562</v>
+        <v>-90561.2347727383</v>
       </c>
       <c r="F22" s="16" t="str">
         <f aca="false">IF(E22&gt;=0,"Sim","Não")</f>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="B23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G17</f>
-        <v>11100.35</v>
+        <v>12810.56</v>
       </c>
       <c r="C23" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A23</f>
@@ -3304,11 +3304,11 @@
       </c>
       <c r="D23" s="12" t="n">
         <f aca="false">B23*C23</f>
-        <v>8951.89516129032</v>
+        <v>10331.0967741935</v>
       </c>
       <c r="E23" s="13" t="n">
         <f aca="false">E22+D23</f>
-        <v>-84698.8162826659</v>
+        <v>-80230.1379985447</v>
       </c>
       <c r="F23" s="16" t="str">
         <f aca="false">IF(E23&gt;=0,"Sim","Não")</f>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="B24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G18</f>
-        <v>15780.9</v>
+        <v>16779.05</v>
       </c>
       <c r="C24" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A24</f>
@@ -3329,11 +3329,11 @@
       </c>
       <c r="D24" s="12" t="n">
         <f aca="false">B24*C24</f>
-        <v>12500.4297047014</v>
+        <v>13291.0882799251</v>
       </c>
       <c r="E24" s="13" t="n">
         <f aca="false">E23+D24</f>
-        <v>-72198.3865779645</v>
+        <v>-66939.0497186196</v>
       </c>
       <c r="F24" s="16" t="str">
         <f aca="false">IF(E24&gt;=0,"Sim","Não")</f>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="B25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G19</f>
-        <v>17465.18</v>
+        <v>18455.26</v>
       </c>
       <c r="C25" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A25</f>
@@ -3354,11 +3354,11 @@
       </c>
       <c r="D25" s="12" t="n">
         <f aca="false">B25*C25</f>
-        <v>13588.7997862379</v>
+        <v>14359.1324648796</v>
       </c>
       <c r="E25" s="13" t="n">
         <f aca="false">E24+D25</f>
-        <v>-58609.5867917266</v>
+        <v>-52579.9172537401</v>
       </c>
       <c r="F25" s="16" t="str">
         <f aca="false">IF(E25&gt;=0,"Sim","Não")</f>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="B26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G20</f>
-        <v>20642.15</v>
+        <v>21030.24</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A26</f>
@@ -3379,11 +3379,11 @@
       </c>
       <c r="D26" s="12" t="n">
         <f aca="false">B26*C26</f>
-        <v>15775.3071249913</v>
+        <v>16071.8963340678</v>
       </c>
       <c r="E26" s="13" t="n">
         <f aca="false">E25+D26</f>
-        <v>-42834.2796667353</v>
+        <v>-36508.0209196723</v>
       </c>
       <c r="F26" s="16" t="str">
         <f aca="false">IF(E26&gt;=0,"Sim","Não")</f>
@@ -3396,7 +3396,7 @@
       </c>
       <c r="B27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G21</f>
-        <v>23185.27</v>
+        <v>23505.03</v>
       </c>
       <c r="C27" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A27</f>
@@ -3404,11 +3404,11 @@
       </c>
       <c r="D27" s="12" t="n">
         <f aca="false">B27*C27</f>
-        <v>17404.0335123917</v>
+        <v>17644.061502401</v>
       </c>
       <c r="E27" s="13" t="n">
         <f aca="false">E26+D27</f>
-        <v>-25430.2461543436</v>
+        <v>-18863.9594172713</v>
       </c>
       <c r="F27" s="16" t="str">
         <f aca="false">IF(E27&gt;=0,"Sim","Não")</f>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G22</f>
-        <v>25553.52</v>
+        <v>25344.17</v>
       </c>
       <c r="C28" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A28</f>
@@ -3429,11 +3429,11 @@
       </c>
       <c r="D28" s="12" t="n">
         <f aca="false">B28*C28</f>
-        <v>18840.9737888107</v>
+        <v>18686.6170558562</v>
       </c>
       <c r="E28" s="13" t="n">
         <f aca="false">E27+D28</f>
-        <v>-6589.27236553283</v>
+        <v>-177.34236141506</v>
       </c>
       <c r="F28" s="16" t="str">
         <f aca="false">IF(E28&gt;=0,"Sim","Não")</f>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G23</f>
-        <v>28111.92</v>
+        <v>27936.65</v>
       </c>
       <c r="C29" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A29</f>
@@ -3454,11 +3454,11 @@
       </c>
       <c r="D29" s="12" t="n">
         <f aca="false">B29*C29</f>
-        <v>20359.0721054537</v>
+        <v>20232.138955106</v>
       </c>
       <c r="E29" s="13" t="n">
         <f aca="false">E28+D29</f>
-        <v>13769.7997399209</v>
+        <v>20054.796593691</v>
       </c>
       <c r="F29" s="16" t="str">
         <f aca="false">IF(E29&gt;=0,"Sim","Não")</f>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B30" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G24</f>
-        <v>31456.01</v>
+        <v>31346.99</v>
       </c>
       <c r="C30" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A30</f>
@@ -3479,11 +3479,11 @@
       </c>
       <c r="D30" s="12" t="n">
         <f aca="false">B30*C30</f>
-        <v>22376.1809832481</v>
+        <v>22298.6297855344</v>
       </c>
       <c r="E30" s="13" t="n">
         <f aca="false">E29+D30</f>
-        <v>36145.980723169</v>
+        <v>42353.4263792254</v>
       </c>
       <c r="F30" s="16" t="str">
         <f aca="false">IF(E30&gt;=0,"Sim","Não")</f>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="B31" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G25</f>
-        <v>34040.97</v>
+        <v>33939.53</v>
       </c>
       <c r="C31" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A31</f>
@@ -3504,11 +3504,11 @@
       </c>
       <c r="D31" s="12" t="n">
         <f aca="false">B31*C31</f>
-        <v>23784.778878397</v>
+        <v>23713.9016980633</v>
       </c>
       <c r="E31" s="13" t="n">
         <f aca="false">E30+D31</f>
-        <v>59930.759601566</v>
+        <v>66067.3280772887</v>
       </c>
       <c r="F31" s="16" t="str">
         <f aca="false">IF(E31&gt;=0,"Sim","Não")</f>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="B32" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G26</f>
-        <v>36654.58</v>
+        <v>36597.94</v>
       </c>
       <c r="C32" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A32</f>
@@ -3529,11 +3529,11 @@
       </c>
       <c r="D32" s="12" t="n">
         <f aca="false">B32*C32</f>
-        <v>25155.9254228279</v>
+        <v>25117.0535651787</v>
       </c>
       <c r="E32" s="13" t="n">
         <f aca="false">E31+D32</f>
-        <v>85086.6850243939</v>
+        <v>91184.3816424674</v>
       </c>
       <c r="F32" s="16" t="str">
         <f aca="false">IF(E32&gt;=0,"Sim","Não")</f>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="B33" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G27</f>
-        <v>38598.09</v>
+        <v>38534.55</v>
       </c>
       <c r="C33" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A33</f>
@@ -3554,11 +3554,11 @@
       </c>
       <c r="D33" s="12" t="n">
         <f aca="false">B33*C33</f>
-        <v>26019.1272431015</v>
+        <v>25976.2946743131</v>
       </c>
       <c r="E33" s="13" t="n">
         <f aca="false">E32+D33</f>
-        <v>111105.812267495</v>
+        <v>117160.676316781</v>
       </c>
       <c r="F33" s="16" t="str">
         <f aca="false">IF(E33&gt;=0,"Sim","Não")</f>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B34" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G28</f>
-        <v>42257.81</v>
+        <v>39699.21</v>
       </c>
       <c r="C34" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A34</f>
@@ -3579,11 +3579,11 @@
       </c>
       <c r="D34" s="12" t="n">
         <f aca="false">B34*C34</f>
-        <v>27980.0673933061</v>
+        <v>26285.9474085622</v>
       </c>
       <c r="E34" s="13" t="n">
         <f aca="false">E33+D34</f>
-        <v>139085.879660802</v>
+        <v>143446.623725343</v>
       </c>
       <c r="F34" s="16" t="str">
         <f aca="false">IF(E34&gt;=0,"Sim","Não")</f>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="B35" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G29</f>
-        <v>44235.79</v>
+        <v>44714.24</v>
       </c>
       <c r="C35" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A35</f>
@@ -3604,11 +3604,11 @@
       </c>
       <c r="D35" s="12" t="n">
         <f aca="false">B35*C35</f>
-        <v>28769.3743496358</v>
+        <v>29080.5411030177</v>
       </c>
       <c r="E35" s="13" t="n">
         <f aca="false">E34+D35</f>
-        <v>167855.254010437</v>
+        <v>172527.16482836</v>
       </c>
       <c r="F35" s="16" t="str">
         <f aca="false">IF(E35&gt;=0,"Sim","Não")</f>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B38" s="24" t="n">
         <f aca="false">SUM(D11:D35)</f>
-        <v>167855.254010437</v>
+        <v>172527.16482836</v>
       </c>
       <c r="C38" s="25" t="str">
         <f aca="false">IF(B38&gt;0,"VIÁVEL: o projeto gera mais do que a taxa exigida",IF(B38&lt;0,"INVIÁVEL: o projeto rende menos que a taxa exigida","EQUILÍBRIO: rende exatamente a taxa exigida"))</f>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="B39" s="26" t="n">
         <f aca="false">IFERROR(IRR(B11:B35),"Não calculável")</f>
-        <v>0.0704388471707102</v>
+        <v>0.0723318571263788</v>
       </c>
       <c r="C39" s="25" t="str">
         <f aca="false">IF(ISNUMBER(B39),IF(B39&gt;B7,"VIÁVEL: TIR maior que a taxa de desconto","INVIÁVEL: TIR menor ou igual à taxa de desconto"),"Sem TIR: o fluxo precisa ter valores negativos E positivos")</f>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="B40" s="26" t="n">
         <f aca="false">IF(ISNUMBER(B39),IF(B6="Mensal",(1+B39)^12-1,B39),"Não calculável")</f>
-        <v>1.26330112699677</v>
+        <v>1.31180127983115</v>
       </c>
       <c r="C40" s="25" t="str">
         <f aca="false">"Compare com a taxa anual de "&amp;ROUND(B5*100,2)&amp;"%"</f>
@@ -3684,11 +3684,11 @@
       </c>
       <c r="B42" s="26" t="n">
         <f aca="false">IF(B41=0,"-",B38/B41)</f>
-        <v>1.64563974520037</v>
+        <v>1.69144279243491</v>
       </c>
       <c r="C42" s="25" t="str">
         <f aca="false">"Para cada R$ 100 de investimento inicial, o projeto gera R$ "&amp;IF(ISNUMBER(B42),ROUND(B42*100,2),"-")&amp;" de VPL acima da taxa exigida"</f>
-        <v>Para cada R$ 100 de investimento inicial, o projeto gera R$ 164.56 de VPL acima da taxa exigida</v>
+        <v>Para cada R$ 100 de investimento inicial, o projeto gera R$ 169.14 de VPL acima da taxa exigida</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B43" s="27" t="n">
         <f aca="false">'Necessidade de Caixa e Payback'!F33</f>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C43" s="25" t="str">
         <f aca="false">"Período em que o saldo acumulado (sem descontar) fica positivo"</f>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="B45" s="24" t="n">
         <f aca="false">'Necessidade de Caixa e Payback'!F32</f>
-        <v>120917.63</v>
+        <v>120917.64</v>
       </c>
       <c r="C45" s="25" t="str">
         <f aca="false">"Dinheiro que os sócios precisam ter para cobrir o pior momento"</f>

</xml_diff>

<commit_message>
Price Core at R$ 1,996, ramp sales and add market sizing
- Core now has a single price of R$ 1,996/month; extra licenses
  (R$ 300) stay in the offer but are not projected.
- New Core clients follow a ladder (3, 5, 7, 10 in months 1-4),
  then grow 5% a month (Premissas B88), with 3% monthly churn.
- Model adds R$ 1,000 acquisition cost per new client, R$ 150
  monthly support per client, ISS above the Simples sublimit and
  Lucro Presumido once RBT12 passes R$ 4.8 mi.
- Template still has only its gray cells filled; Memoria de
  Calculo gains a Mercado TAM SAM SOM sheet.
- New Precept_Pesquisa_de_Mercado (beachhead, TAM, SAM, SOM with
  pessimistic/central/optimistic ranges).
- Ficha, planning document, pitch slides 10 and 16 and the Matriz
  updated to the new numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016kLWp3PkVdryYcjkVkag3m
</commit_message>
<xml_diff>
--- a/precept-financeiro/Planilha_Financeira_Precept.xlsx
+++ b/precept-financeiro/Planilha_Financeira_Precept.xlsx
@@ -1308,21 +1308,21 @@
         <v>5988</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>1479.9</v>
+        <v>4767.9</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>12000</v>
       </c>
       <c r="E6" s="12" t="n">
         <f aca="false">B6-C6-D6</f>
-        <v>-7491.9</v>
+        <v>-10779.9</v>
       </c>
       <c r="F6" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="13" t="n">
         <f aca="false">E6-F6</f>
-        <v>-7491.9</v>
+        <v>-10779.9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1330,24 +1330,24 @@
         <v>2</v>
       </c>
       <c r="B7" s="11" t="n">
-        <v>8982</v>
+        <v>15968</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>2219.85</v>
+        <v>9714.4</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>12000</v>
       </c>
       <c r="E7" s="12" t="n">
         <f aca="false">B7-C7-D7</f>
-        <v>-5237.85</v>
+        <v>-5746.4</v>
       </c>
       <c r="F7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="13" t="n">
         <f aca="false">E7-F7</f>
-        <v>-5237.85</v>
+        <v>-5746.4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1355,24 +1355,24 @@
         <v>3</v>
       </c>
       <c r="B8" s="11" t="n">
-        <v>13473</v>
+        <v>29940</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>3329.78</v>
+        <v>15839.5</v>
       </c>
       <c r="D8" s="11" t="n">
         <v>12000</v>
       </c>
       <c r="E8" s="12" t="n">
         <f aca="false">B8-C8-D8</f>
-        <v>-1856.78</v>
+        <v>2100.5</v>
       </c>
       <c r="F8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="13" t="n">
         <f aca="false">E8-F8</f>
-        <v>-1856.78</v>
+        <v>2100.5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1380,24 +1380,24 @@
         <v>4</v>
       </c>
       <c r="B9" s="11" t="n">
-        <v>24967</v>
+        <v>57901</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>10156.03</v>
+        <v>30923.82</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>18116.92</v>
+        <v>26185.75</v>
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">B9-C9-D9</f>
-        <v>-3305.95</v>
+        <v>791.43</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="13" t="n">
         <f aca="false">E9-F9</f>
-        <v>-3305.95</v>
+        <v>791.43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1405,24 +1405,24 @@
         <v>5</v>
       </c>
       <c r="B10" s="11" t="n">
-        <v>29458</v>
+        <v>77861</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>11265.95</v>
+        <v>38507.3</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>19217.21</v>
+        <v>31075.95</v>
       </c>
       <c r="E10" s="12" t="n">
         <f aca="false">B10-C10-D10</f>
-        <v>-1025.16</v>
+        <v>8277.75</v>
       </c>
       <c r="F10" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="13" t="n">
         <f aca="false">E10-F10</f>
-        <v>-1025.16</v>
+        <v>8277.75</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1430,24 +1430,24 @@
         <v>6</v>
       </c>
       <c r="B11" s="11" t="n">
-        <v>60952</v>
+        <v>125822</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>30336.88</v>
+        <v>63883.58</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>26933.24</v>
+        <v>42826.39</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">B11-C11-D11</f>
-        <v>3681.88</v>
+        <v>19112.03</v>
       </c>
       <c r="F11" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="13" t="n">
         <f aca="false">E11-F11</f>
-        <v>3681.88</v>
+        <v>19112.03</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1455,24 +1455,24 @@
         <v>7</v>
       </c>
       <c r="B12" s="11" t="n">
-        <v>35446</v>
+        <v>117781</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>13185.46</v>
+        <v>53501.9</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>20684.27</v>
+        <v>40856.35</v>
       </c>
       <c r="E12" s="12" t="n">
         <f aca="false">B12-C12-D12</f>
-        <v>1576.27</v>
+        <v>23422.75</v>
       </c>
       <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="13" t="n">
         <f aca="false">E12-F12</f>
-        <v>1576.27</v>
+        <v>23422.75</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1480,24 +1480,24 @@
         <v>8</v>
       </c>
       <c r="B13" s="11" t="n">
-        <v>66940</v>
+        <v>165742</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>32473.39</v>
+        <v>79095.96</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>28400.3</v>
+        <v>52606.79</v>
       </c>
       <c r="E13" s="12" t="n">
         <f aca="false">B13-C13-D13</f>
-        <v>6066.31</v>
+        <v>34039.25</v>
       </c>
       <c r="F13" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">E13-F13</f>
-        <v>6066.31</v>
+        <v>34039.25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1505,24 +1505,24 @@
         <v>9</v>
       </c>
       <c r="B14" s="11" t="n">
-        <v>51431</v>
+        <v>167698</v>
       </c>
       <c r="C14" s="11" t="n">
-        <v>21468.56</v>
+        <v>75207.39</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>24600.6</v>
+        <v>53086.01</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">B14-C14-D14</f>
-        <v>5361.84</v>
+        <v>39404.6</v>
       </c>
       <c r="F14" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">E14-F14</f>
-        <v>5361.84</v>
+        <v>39404.6</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1530,24 +1530,24 @@
         <v>10</v>
       </c>
       <c r="B15" s="11" t="n">
-        <v>74425</v>
+        <v>209654</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>34750.33</v>
+        <v>95573.59</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>30234.12</v>
+        <v>63365.23</v>
       </c>
       <c r="E15" s="12" t="n">
         <f aca="false">B15-C15-D15</f>
-        <v>9440.55</v>
+        <v>50715.18</v>
       </c>
       <c r="F15" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="13" t="n">
         <f aca="false">E15-F15</f>
-        <v>9440.55</v>
+        <v>50715.18</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1555,24 +1555,24 @@
         <v>11</v>
       </c>
       <c r="B16" s="11" t="n">
-        <v>58916</v>
+        <v>211610</v>
       </c>
       <c r="C16" s="11" t="n">
-        <v>23690.15</v>
+        <v>91475.04</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>26434.42</v>
+        <v>63844.45</v>
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">B16-C16-D16</f>
-        <v>8791.43</v>
+        <v>56290.51</v>
       </c>
       <c r="F16" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="13" t="n">
         <f aca="false">E16-F16</f>
-        <v>8791.43</v>
+        <v>56290.51</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1580,24 +1580,24 @@
         <v>12</v>
       </c>
       <c r="B17" s="11" t="n">
-        <v>81910</v>
+        <v>255562</v>
       </c>
       <c r="C17" s="11" t="n">
-        <v>37031.49</v>
+        <v>113561.27</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>32067.95</v>
+        <v>74612.69</v>
       </c>
       <c r="E17" s="12" t="n">
         <f aca="false">B17-C17-D17</f>
-        <v>12810.56</v>
+        <v>67388.04</v>
       </c>
       <c r="F17" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G17" s="13" t="n">
         <f aca="false">E17-F17</f>
-        <v>12810.56</v>
+        <v>67388.04</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1605,24 +1605,24 @@
         <v>13</v>
       </c>
       <c r="B18" s="11" t="n">
-        <v>114895</v>
+        <v>305513</v>
       </c>
       <c r="C18" s="11" t="n">
-        <v>57966.67</v>
+        <v>142470.3</v>
       </c>
       <c r="D18" s="11" t="n">
-        <v>40149.28</v>
+        <v>86850.69</v>
       </c>
       <c r="E18" s="12" t="n">
         <f aca="false">B18-C18-D18</f>
-        <v>16779.05</v>
+        <v>76192.01</v>
       </c>
       <c r="F18" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="13" t="n">
         <f aca="false">E18-F18</f>
-        <v>16779.05</v>
+        <v>76192.01</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1630,24 +1630,24 @@
         <v>14</v>
       </c>
       <c r="B19" s="11" t="n">
-        <v>119386</v>
+        <v>327469</v>
       </c>
       <c r="C19" s="11" t="n">
-        <v>59681.17</v>
+        <v>150698.24</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>41249.57</v>
+        <v>92229.91</v>
       </c>
       <c r="E19" s="12" t="n">
         <f aca="false">B19-C19-D19</f>
-        <v>18455.26</v>
+        <v>84540.85</v>
       </c>
       <c r="F19" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G19" s="13" t="n">
         <f aca="false">E19-F19</f>
-        <v>18455.26</v>
+        <v>84540.85</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1655,24 +1655,24 @@
         <v>15</v>
       </c>
       <c r="B20" s="11" t="n">
-        <v>125374</v>
+        <v>353417</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>61627.13</v>
+        <v>162015.62</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>42716.63</v>
+        <v>98587.17</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">B20-C20-D20</f>
-        <v>21030.24</v>
+        <v>92814.21</v>
       </c>
       <c r="F20" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="13" t="n">
         <f aca="false">E20-F20</f>
-        <v>21030.24</v>
+        <v>92814.21</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1680,24 +1680,24 @@
         <v>16</v>
       </c>
       <c r="B21" s="11" t="n">
-        <v>131362</v>
+        <v>381361</v>
       </c>
       <c r="C21" s="11" t="n">
-        <v>63673.28</v>
+        <v>174086.99</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>44183.69</v>
+        <v>105433.45</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">B21-C21-D21</f>
-        <v>23505.03</v>
+        <v>101840.56</v>
       </c>
       <c r="F21" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">E21-F21</f>
-        <v>23505.03</v>
+        <v>101840.56</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1705,24 +1705,24 @@
         <v>17</v>
       </c>
       <c r="B22" s="11" t="n">
-        <v>135853</v>
+        <v>409305</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>65224.84</v>
+        <v>185984.46</v>
       </c>
       <c r="D22" s="11" t="n">
-        <v>45283.99</v>
+        <v>112279.73</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">B22-C22-D22</f>
-        <v>25344.17</v>
+        <v>111040.81</v>
       </c>
       <c r="F22" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">E22-F22</f>
-        <v>25344.17</v>
+        <v>111040.81</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1730,24 +1730,24 @@
         <v>18</v>
       </c>
       <c r="B23" s="11" t="n">
-        <v>141841</v>
+        <v>439245</v>
       </c>
       <c r="C23" s="11" t="n">
-        <v>67153.3</v>
+        <v>198485.68</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>46751.05</v>
+        <v>119615.03</v>
       </c>
       <c r="E23" s="12" t="n">
         <f aca="false">B23-C23-D23</f>
-        <v>27936.65</v>
+        <v>121144.29</v>
       </c>
       <c r="F23" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">E23-F23</f>
-        <v>27936.65</v>
+        <v>121144.29</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1755,24 +1755,24 @@
         <v>19</v>
       </c>
       <c r="B24" s="11" t="n">
-        <v>157826</v>
+        <v>477186</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>75811.64</v>
+        <v>217308.63</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>50667.37</v>
+        <v>128910.57</v>
       </c>
       <c r="E24" s="12" t="n">
         <f aca="false">B24-C24-D24</f>
-        <v>31346.99</v>
+        <v>130966.8</v>
       </c>
       <c r="F24" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="13" t="n">
         <f aca="false">E24-F24</f>
-        <v>31346.99</v>
+        <v>130966.8</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1780,24 +1780,24 @@
         <v>20</v>
       </c>
       <c r="B25" s="11" t="n">
-        <v>163814</v>
+        <v>509122</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>77740.04</v>
+        <v>228404.73</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>52134.43</v>
+        <v>136734.89</v>
       </c>
       <c r="E25" s="12" t="n">
         <f aca="false">B25-C25-D25</f>
-        <v>33939.53</v>
+        <v>143982.38</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">E25-F25</f>
-        <v>33939.53</v>
+        <v>143982.38</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1805,24 +1805,24 @@
         <v>21</v>
       </c>
       <c r="B26" s="11" t="n">
-        <v>169802</v>
+        <v>541058</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>79602.57</v>
+        <v>247257.54</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>53601.49</v>
+        <v>144559.21</v>
       </c>
       <c r="E26" s="12" t="n">
         <f aca="false">B26-C26-D26</f>
-        <v>36597.94</v>
+        <v>149241.25</v>
       </c>
       <c r="F26" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G26" s="13" t="n">
         <f aca="false">E26-F26</f>
-        <v>36597.94</v>
+        <v>149241.25</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1830,24 +1830,24 @@
         <v>22</v>
       </c>
       <c r="B27" s="11" t="n">
-        <v>174293</v>
+        <v>574990</v>
       </c>
       <c r="C27" s="11" t="n">
-        <v>81056.66</v>
+        <v>267014.38</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>54701.79</v>
+        <v>152872.55</v>
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">B27-C27-D27</f>
-        <v>38534.55</v>
+        <v>155103.07</v>
       </c>
       <c r="F27" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="13" t="n">
         <f aca="false">E27-F27</f>
-        <v>38534.55</v>
+        <v>155103.07</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1855,24 +1855,24 @@
         <v>23</v>
       </c>
       <c r="B28" s="11" t="n">
-        <v>153278</v>
+        <v>580921</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>64025.68</v>
+        <v>265812.37</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>49553.11</v>
+        <v>154325.65</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">B28-C28-D28</f>
-        <v>39699.21</v>
+        <v>160782.98</v>
       </c>
       <c r="F28" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="13" t="n">
         <f aca="false">E28-F28</f>
-        <v>39699.21</v>
+        <v>160782.98</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1880,24 +1880,24 @@
         <v>24</v>
       </c>
       <c r="B29" s="11" t="n">
-        <v>187766</v>
+        <v>648842</v>
       </c>
       <c r="C29" s="11" t="n">
-        <v>85049.09</v>
+        <v>270968.48</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>58002.67</v>
+        <v>170966.29</v>
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">B29-C29-D29</f>
-        <v>44714.24</v>
+        <v>206907.23</v>
       </c>
       <c r="F29" s="11" t="n">
         <v>0</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">E29-F29</f>
-        <v>44714.24</v>
+        <v>206907.23</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1906,19 +1906,19 @@
       </c>
       <c r="B30" s="13" t="n">
         <f aca="false">SUM(B5:B29)</f>
-        <v>2288378</v>
+        <v>6989956</v>
       </c>
       <c r="C30" s="13" t="n">
         <f aca="false">SUM(C5:C29)</f>
-        <v>1059999.84</v>
+        <v>3182559.07</v>
       </c>
       <c r="D30" s="13" t="n">
         <f aca="false">SUM(D5:D29)</f>
-        <v>841684.1</v>
+        <v>1987824.75</v>
       </c>
       <c r="E30" s="13" t="n">
         <f aca="false">SUM(E5:E29)</f>
-        <v>386694.06</v>
+        <v>1819572.18</v>
       </c>
       <c r="F30" s="13" t="n">
         <f aca="false">SUM(F5:F29)</f>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="G30" s="13" t="n">
         <f aca="false">SUM(G5:G29)</f>
-        <v>284694.06</v>
+        <v>1717572.18</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="C6" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C6</f>
-        <v>1479.9</v>
+        <v>4767.9</v>
       </c>
       <c r="D6" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D6</f>
@@ -2059,11 +2059,11 @@
       </c>
       <c r="F6" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G6</f>
-        <v>-7491.9</v>
+        <v>-10779.9</v>
       </c>
       <c r="G6" s="13" t="n">
         <f aca="false">G5+F6</f>
-        <v>-109491.9</v>
+        <v>-112779.9</v>
       </c>
       <c r="H6" s="16" t="str">
         <f aca="false">IF(G6&gt;=0,"Sim","Não")</f>
@@ -2076,11 +2076,11 @@
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B7</f>
-        <v>8982</v>
+        <v>15968</v>
       </c>
       <c r="C7" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C7</f>
-        <v>2219.85</v>
+        <v>9714.4</v>
       </c>
       <c r="D7" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D7</f>
@@ -2092,11 +2092,11 @@
       </c>
       <c r="F7" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G7</f>
-        <v>-5237.85</v>
+        <v>-5746.4</v>
       </c>
       <c r="G7" s="13" t="n">
         <f aca="false">G6+F7</f>
-        <v>-114729.75</v>
+        <v>-118526.3</v>
       </c>
       <c r="H7" s="16" t="str">
         <f aca="false">IF(G7&gt;=0,"Sim","Não")</f>
@@ -2109,11 +2109,11 @@
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B8</f>
-        <v>13473</v>
+        <v>29940</v>
       </c>
       <c r="C8" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C8</f>
-        <v>3329.78</v>
+        <v>15839.5</v>
       </c>
       <c r="D8" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D8</f>
@@ -2125,11 +2125,11 @@
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G8</f>
-        <v>-1856.78</v>
+        <v>2100.5</v>
       </c>
       <c r="G8" s="13" t="n">
         <f aca="false">G7+F8</f>
-        <v>-116586.53</v>
+        <v>-116425.8</v>
       </c>
       <c r="H8" s="16" t="str">
         <f aca="false">IF(G8&gt;=0,"Sim","Não")</f>
@@ -2142,15 +2142,15 @@
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B9</f>
-        <v>24967</v>
+        <v>57901</v>
       </c>
       <c r="C9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C9</f>
-        <v>10156.03</v>
+        <v>30923.82</v>
       </c>
       <c r="D9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D9</f>
-        <v>18116.92</v>
+        <v>26185.75</v>
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F9</f>
@@ -2158,11 +2158,11 @@
       </c>
       <c r="F9" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G9</f>
-        <v>-3305.95</v>
+        <v>791.43</v>
       </c>
       <c r="G9" s="13" t="n">
         <f aca="false">G8+F9</f>
-        <v>-119892.48</v>
+        <v>-115634.37</v>
       </c>
       <c r="H9" s="16" t="str">
         <f aca="false">IF(G9&gt;=0,"Sim","Não")</f>
@@ -2175,15 +2175,15 @@
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B10</f>
-        <v>29458</v>
+        <v>77861</v>
       </c>
       <c r="C10" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C10</f>
-        <v>11265.95</v>
+        <v>38507.3</v>
       </c>
       <c r="D10" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D10</f>
-        <v>19217.21</v>
+        <v>31075.95</v>
       </c>
       <c r="E10" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F10</f>
@@ -2191,11 +2191,11 @@
       </c>
       <c r="F10" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G10</f>
-        <v>-1025.16</v>
+        <v>8277.75</v>
       </c>
       <c r="G10" s="13" t="n">
         <f aca="false">G9+F10</f>
-        <v>-120917.64</v>
+        <v>-107356.62</v>
       </c>
       <c r="H10" s="16" t="str">
         <f aca="false">IF(G10&gt;=0,"Sim","Não")</f>
@@ -2208,15 +2208,15 @@
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B11</f>
-        <v>60952</v>
+        <v>125822</v>
       </c>
       <c r="C11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C11</f>
-        <v>30336.88</v>
+        <v>63883.58</v>
       </c>
       <c r="D11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D11</f>
-        <v>26933.24</v>
+        <v>42826.39</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F11</f>
@@ -2224,11 +2224,11 @@
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G11</f>
-        <v>3681.88</v>
+        <v>19112.03</v>
       </c>
       <c r="G11" s="13" t="n">
         <f aca="false">G10+F11</f>
-        <v>-117235.76</v>
+        <v>-88244.59</v>
       </c>
       <c r="H11" s="16" t="str">
         <f aca="false">IF(G11&gt;=0,"Sim","Não")</f>
@@ -2241,15 +2241,15 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B12</f>
-        <v>35446</v>
+        <v>117781</v>
       </c>
       <c r="C12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C12</f>
-        <v>13185.46</v>
+        <v>53501.9</v>
       </c>
       <c r="D12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D12</f>
-        <v>20684.27</v>
+        <v>40856.35</v>
       </c>
       <c r="E12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F12</f>
@@ -2257,11 +2257,11 @@
       </c>
       <c r="F12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G12</f>
-        <v>1576.27</v>
+        <v>23422.75</v>
       </c>
       <c r="G12" s="13" t="n">
         <f aca="false">G11+F12</f>
-        <v>-115659.49</v>
+        <v>-64821.84</v>
       </c>
       <c r="H12" s="16" t="str">
         <f aca="false">IF(G12&gt;=0,"Sim","Não")</f>
@@ -2274,15 +2274,15 @@
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B13</f>
-        <v>66940</v>
+        <v>165742</v>
       </c>
       <c r="C13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C13</f>
-        <v>32473.39</v>
+        <v>79095.96</v>
       </c>
       <c r="D13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D13</f>
-        <v>28400.3</v>
+        <v>52606.79</v>
       </c>
       <c r="E13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F13</f>
@@ -2290,11 +2290,11 @@
       </c>
       <c r="F13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G13</f>
-        <v>6066.31</v>
+        <v>34039.25</v>
       </c>
       <c r="G13" s="13" t="n">
         <f aca="false">G12+F13</f>
-        <v>-109593.18</v>
+        <v>-30782.59</v>
       </c>
       <c r="H13" s="16" t="str">
         <f aca="false">IF(G13&gt;=0,"Sim","Não")</f>
@@ -2307,15 +2307,15 @@
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B14</f>
-        <v>51431</v>
+        <v>167698</v>
       </c>
       <c r="C14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C14</f>
-        <v>21468.56</v>
+        <v>75207.39</v>
       </c>
       <c r="D14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D14</f>
-        <v>24600.6</v>
+        <v>53086.01</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F14</f>
@@ -2323,15 +2323,15 @@
       </c>
       <c r="F14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G14</f>
-        <v>5361.84</v>
+        <v>39404.6</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">G13+F14</f>
-        <v>-104231.34</v>
+        <v>8622.01</v>
       </c>
       <c r="H14" s="16" t="str">
         <f aca="false">IF(G14&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2340,15 +2340,15 @@
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B15</f>
-        <v>74425</v>
+        <v>209654</v>
       </c>
       <c r="C15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C15</f>
-        <v>34750.33</v>
+        <v>95573.59</v>
       </c>
       <c r="D15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D15</f>
-        <v>30234.12</v>
+        <v>63365.23</v>
       </c>
       <c r="E15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F15</f>
@@ -2356,15 +2356,15 @@
       </c>
       <c r="F15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G15</f>
-        <v>9440.55</v>
+        <v>50715.18</v>
       </c>
       <c r="G15" s="13" t="n">
         <f aca="false">G14+F15</f>
-        <v>-94790.79</v>
+        <v>59337.19</v>
       </c>
       <c r="H15" s="16" t="str">
         <f aca="false">IF(G15&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2373,15 +2373,15 @@
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B16</f>
-        <v>58916</v>
+        <v>211610</v>
       </c>
       <c r="C16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C16</f>
-        <v>23690.15</v>
+        <v>91475.04</v>
       </c>
       <c r="D16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D16</f>
-        <v>26434.42</v>
+        <v>63844.45</v>
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F16</f>
@@ -2389,15 +2389,15 @@
       </c>
       <c r="F16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G16</f>
-        <v>8791.43</v>
+        <v>56290.51</v>
       </c>
       <c r="G16" s="13" t="n">
         <f aca="false">G15+F16</f>
-        <v>-85999.36</v>
+        <v>115627.7</v>
       </c>
       <c r="H16" s="16" t="str">
         <f aca="false">IF(G16&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2406,15 +2406,15 @@
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B17</f>
-        <v>81910</v>
+        <v>255562</v>
       </c>
       <c r="C17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C17</f>
-        <v>37031.49</v>
+        <v>113561.27</v>
       </c>
       <c r="D17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D17</f>
-        <v>32067.95</v>
+        <v>74612.69</v>
       </c>
       <c r="E17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F17</f>
@@ -2422,15 +2422,15 @@
       </c>
       <c r="F17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G17</f>
-        <v>12810.56</v>
+        <v>67388.04</v>
       </c>
       <c r="G17" s="13" t="n">
         <f aca="false">G16+F17</f>
-        <v>-73188.8</v>
+        <v>183015.74</v>
       </c>
       <c r="H17" s="16" t="str">
         <f aca="false">IF(G17&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2439,15 +2439,15 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B18</f>
-        <v>114895</v>
+        <v>305513</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C18</f>
-        <v>57966.67</v>
+        <v>142470.3</v>
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D18</f>
-        <v>40149.28</v>
+        <v>86850.69</v>
       </c>
       <c r="E18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F18</f>
@@ -2455,15 +2455,15 @@
       </c>
       <c r="F18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G18</f>
-        <v>16779.05</v>
+        <v>76192.01</v>
       </c>
       <c r="G18" s="13" t="n">
         <f aca="false">G17+F18</f>
-        <v>-56409.75</v>
+        <v>259207.75</v>
       </c>
       <c r="H18" s="16" t="str">
         <f aca="false">IF(G18&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2472,15 +2472,15 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B19</f>
-        <v>119386</v>
+        <v>327469</v>
       </c>
       <c r="C19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C19</f>
-        <v>59681.17</v>
+        <v>150698.24</v>
       </c>
       <c r="D19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D19</f>
-        <v>41249.57</v>
+        <v>92229.91</v>
       </c>
       <c r="E19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F19</f>
@@ -2488,15 +2488,15 @@
       </c>
       <c r="F19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G19</f>
-        <v>18455.26</v>
+        <v>84540.85</v>
       </c>
       <c r="G19" s="13" t="n">
         <f aca="false">G18+F19</f>
-        <v>-37954.49</v>
+        <v>343748.6</v>
       </c>
       <c r="H19" s="16" t="str">
         <f aca="false">IF(G19&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2505,15 +2505,15 @@
       </c>
       <c r="B20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B20</f>
-        <v>125374</v>
+        <v>353417</v>
       </c>
       <c r="C20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C20</f>
-        <v>61627.13</v>
+        <v>162015.62</v>
       </c>
       <c r="D20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D20</f>
-        <v>42716.63</v>
+        <v>98587.17</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F20</f>
@@ -2521,15 +2521,15 @@
       </c>
       <c r="F20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G20</f>
-        <v>21030.24</v>
+        <v>92814.21</v>
       </c>
       <c r="G20" s="13" t="n">
         <f aca="false">G19+F20</f>
-        <v>-16924.25</v>
+        <v>436562.81</v>
       </c>
       <c r="H20" s="16" t="str">
         <f aca="false">IF(G20&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2538,15 +2538,15 @@
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B21</f>
-        <v>131362</v>
+        <v>381361</v>
       </c>
       <c r="C21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C21</f>
-        <v>63673.28</v>
+        <v>174086.99</v>
       </c>
       <c r="D21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D21</f>
-        <v>44183.69</v>
+        <v>105433.45</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F21</f>
@@ -2554,11 +2554,11 @@
       </c>
       <c r="F21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G21</f>
-        <v>23505.03</v>
+        <v>101840.56</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">G20+F21</f>
-        <v>6580.77999999999</v>
+        <v>538403.37</v>
       </c>
       <c r="H21" s="16" t="str">
         <f aca="false">IF(G21&gt;=0,"Sim","Não")</f>
@@ -2571,15 +2571,15 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B22</f>
-        <v>135853</v>
+        <v>409305</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C22</f>
-        <v>65224.84</v>
+        <v>185984.46</v>
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D22</f>
-        <v>45283.99</v>
+        <v>112279.73</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F22</f>
@@ -2587,11 +2587,11 @@
       </c>
       <c r="F22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G22</f>
-        <v>25344.17</v>
+        <v>111040.81</v>
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">G21+F22</f>
-        <v>31924.95</v>
+        <v>649444.18</v>
       </c>
       <c r="H22" s="16" t="str">
         <f aca="false">IF(G22&gt;=0,"Sim","Não")</f>
@@ -2604,15 +2604,15 @@
       </c>
       <c r="B23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B23</f>
-        <v>141841</v>
+        <v>439245</v>
       </c>
       <c r="C23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C23</f>
-        <v>67153.3</v>
+        <v>198485.68</v>
       </c>
       <c r="D23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D23</f>
-        <v>46751.05</v>
+        <v>119615.03</v>
       </c>
       <c r="E23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F23</f>
@@ -2620,11 +2620,11 @@
       </c>
       <c r="F23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G23</f>
-        <v>27936.65</v>
+        <v>121144.29</v>
       </c>
       <c r="G23" s="13" t="n">
         <f aca="false">G22+F23</f>
-        <v>59861.6</v>
+        <v>770588.47</v>
       </c>
       <c r="H23" s="16" t="str">
         <f aca="false">IF(G23&gt;=0,"Sim","Não")</f>
@@ -2637,15 +2637,15 @@
       </c>
       <c r="B24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B24</f>
-        <v>157826</v>
+        <v>477186</v>
       </c>
       <c r="C24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C24</f>
-        <v>75811.64</v>
+        <v>217308.63</v>
       </c>
       <c r="D24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D24</f>
-        <v>50667.37</v>
+        <v>128910.57</v>
       </c>
       <c r="E24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F24</f>
@@ -2653,11 +2653,11 @@
       </c>
       <c r="F24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G24</f>
-        <v>31346.99</v>
+        <v>130966.8</v>
       </c>
       <c r="G24" s="13" t="n">
         <f aca="false">G23+F24</f>
-        <v>91208.59</v>
+        <v>901555.27</v>
       </c>
       <c r="H24" s="16" t="str">
         <f aca="false">IF(G24&gt;=0,"Sim","Não")</f>
@@ -2670,15 +2670,15 @@
       </c>
       <c r="B25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B25</f>
-        <v>163814</v>
+        <v>509122</v>
       </c>
       <c r="C25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C25</f>
-        <v>77740.04</v>
+        <v>228404.73</v>
       </c>
       <c r="D25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D25</f>
-        <v>52134.43</v>
+        <v>136734.89</v>
       </c>
       <c r="E25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F25</f>
@@ -2686,11 +2686,11 @@
       </c>
       <c r="F25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G25</f>
-        <v>33939.53</v>
+        <v>143982.38</v>
       </c>
       <c r="G25" s="13" t="n">
         <f aca="false">G24+F25</f>
-        <v>125148.12</v>
+        <v>1045537.65</v>
       </c>
       <c r="H25" s="16" t="str">
         <f aca="false">IF(G25&gt;=0,"Sim","Não")</f>
@@ -2703,15 +2703,15 @@
       </c>
       <c r="B26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B26</f>
-        <v>169802</v>
+        <v>541058</v>
       </c>
       <c r="C26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C26</f>
-        <v>79602.57</v>
+        <v>247257.54</v>
       </c>
       <c r="D26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D26</f>
-        <v>53601.49</v>
+        <v>144559.21</v>
       </c>
       <c r="E26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F26</f>
@@ -2719,11 +2719,11 @@
       </c>
       <c r="F26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G26</f>
-        <v>36597.94</v>
+        <v>149241.25</v>
       </c>
       <c r="G26" s="13" t="n">
         <f aca="false">G25+F26</f>
-        <v>161746.06</v>
+        <v>1194778.9</v>
       </c>
       <c r="H26" s="16" t="str">
         <f aca="false">IF(G26&gt;=0,"Sim","Não")</f>
@@ -2736,15 +2736,15 @@
       </c>
       <c r="B27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B27</f>
-        <v>174293</v>
+        <v>574990</v>
       </c>
       <c r="C27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C27</f>
-        <v>81056.66</v>
+        <v>267014.38</v>
       </c>
       <c r="D27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D27</f>
-        <v>54701.79</v>
+        <v>152872.55</v>
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F27</f>
@@ -2752,11 +2752,11 @@
       </c>
       <c r="F27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G27</f>
-        <v>38534.55</v>
+        <v>155103.07</v>
       </c>
       <c r="G27" s="13" t="n">
         <f aca="false">G26+F27</f>
-        <v>200280.61</v>
+        <v>1349881.97</v>
       </c>
       <c r="H27" s="16" t="str">
         <f aca="false">IF(G27&gt;=0,"Sim","Não")</f>
@@ -2769,15 +2769,15 @@
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B28</f>
-        <v>153278</v>
+        <v>580921</v>
       </c>
       <c r="C28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C28</f>
-        <v>64025.68</v>
+        <v>265812.37</v>
       </c>
       <c r="D28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D28</f>
-        <v>49553.11</v>
+        <v>154325.65</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F28</f>
@@ -2785,11 +2785,11 @@
       </c>
       <c r="F28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G28</f>
-        <v>39699.21</v>
+        <v>160782.98</v>
       </c>
       <c r="G28" s="13" t="n">
         <f aca="false">G27+F28</f>
-        <v>239979.82</v>
+        <v>1510664.95</v>
       </c>
       <c r="H28" s="16" t="str">
         <f aca="false">IF(G28&gt;=0,"Sim","Não")</f>
@@ -2802,15 +2802,15 @@
       </c>
       <c r="B29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!B29</f>
-        <v>187766</v>
+        <v>648842</v>
       </c>
       <c r="C29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!C29</f>
-        <v>85049.09</v>
+        <v>270968.48</v>
       </c>
       <c r="D29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!D29</f>
-        <v>58002.67</v>
+        <v>170966.29</v>
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!F29</f>
@@ -2818,11 +2818,11 @@
       </c>
       <c r="F29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G29</f>
-        <v>44714.24</v>
+        <v>206907.23</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">G28+F29</f>
-        <v>284694.06</v>
+        <v>1717572.18</v>
       </c>
       <c r="H29" s="16" t="str">
         <f aca="false">IF(G29&gt;=0,"Sim","Não")</f>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="F32" s="17" t="n">
         <f aca="false">MAX(0,-MIN(G5:G29))</f>
-        <v>120917.64</v>
+        <v>118526.3</v>
       </c>
       <c r="G32" s="18" t="s">
         <v>45</v>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="F33" s="19" t="n">
         <f aca="false">IFERROR(INDEX(A5:A29,MATCH("Sim",H5:H29,0)),"Não recupera")</f>
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G33" s="18" t="s">
         <v>47</v>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G6</f>
-        <v>-7491.9</v>
+        <v>-10779.9</v>
       </c>
       <c r="C12" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A12</f>
@@ -3029,11 +3029,11 @@
       </c>
       <c r="D12" s="12" t="n">
         <f aca="false">B12*C12</f>
-        <v>-7358.79714957759</v>
+        <v>-10588.3817713439</v>
       </c>
       <c r="E12" s="13" t="n">
         <f aca="false">E11+D12</f>
-        <v>-109358.797149578</v>
+        <v>-112588.381771344</v>
       </c>
       <c r="F12" s="16" t="str">
         <f aca="false">IF(E12&gt;=0,"Sim","Não")</f>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G7</f>
-        <v>-5237.85</v>
+        <v>-5746.4</v>
       </c>
       <c r="C13" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A13</f>
@@ -3054,11 +3054,11 @@
       </c>
       <c r="D13" s="12" t="n">
         <f aca="false">B13*C13</f>
-        <v>-5053.38952995787</v>
+        <v>-5544.03001135006</v>
       </c>
       <c r="E13" s="13" t="n">
         <f aca="false">E12+D13</f>
-        <v>-114412.186679535</v>
+        <v>-118132.411782694</v>
       </c>
       <c r="F13" s="16" t="str">
         <f aca="false">IF(E13&gt;=0,"Sim","Não")</f>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="B14" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G8</f>
-        <v>-1856.78</v>
+        <v>2100.5</v>
       </c>
       <c r="C14" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A14</f>
@@ -3079,11 +3079,11 @@
       </c>
       <c r="D14" s="12" t="n">
         <f aca="false">B14*C14</f>
-        <v>-1759.56383936708</v>
+        <v>1990.52329548496</v>
       </c>
       <c r="E14" s="13" t="n">
         <f aca="false">E13+D14</f>
-        <v>-116171.750518903</v>
+        <v>-116141.888487209</v>
       </c>
       <c r="F14" s="16" t="str">
         <f aca="false">IF(E14&gt;=0,"Sim","Não")</f>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G9</f>
-        <v>-3305.95</v>
+        <v>791.43</v>
       </c>
       <c r="C15" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A15</f>
@@ -3104,11 +3104,11 @@
       </c>
       <c r="D15" s="12" t="n">
         <f aca="false">B15*C15</f>
-        <v>-3077.19996756395</v>
+        <v>736.66824069606</v>
       </c>
       <c r="E15" s="13" t="n">
         <f aca="false">E14+D15</f>
-        <v>-119248.950486466</v>
+        <v>-115405.220246513</v>
       </c>
       <c r="F15" s="16" t="str">
         <f aca="false">IF(E15&gt;=0,"Sim","Não")</f>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G10</f>
-        <v>-1025.16</v>
+        <v>8277.75</v>
       </c>
       <c r="C16" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A16</f>
@@ -3129,11 +3129,11 @@
       </c>
       <c r="D16" s="12" t="n">
         <f aca="false">B16*C16</f>
-        <v>-937.272662818201</v>
+        <v>7568.09550181763</v>
       </c>
       <c r="E16" s="13" t="n">
         <f aca="false">E15+D16</f>
-        <v>-120186.223149285</v>
+        <v>-107837.124744695</v>
       </c>
       <c r="F16" s="16" t="str">
         <f aca="false">IF(E16&gt;=0,"Sim","Não")</f>
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G11</f>
-        <v>3681.88</v>
+        <v>19112.03</v>
       </c>
       <c r="C17" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A17</f>
@@ -3154,11 +3154,11 @@
       </c>
       <c r="D17" s="12" t="n">
         <f aca="false">B17*C17</f>
-        <v>3306.42584713171</v>
+        <v>17163.1096024739</v>
       </c>
       <c r="E17" s="13" t="n">
         <f aca="false">E16+D17</f>
-        <v>-116879.797302153</v>
+        <v>-90674.0151422214</v>
       </c>
       <c r="F17" s="16" t="str">
         <f aca="false">IF(E17&gt;=0,"Sim","Não")</f>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G12</f>
-        <v>1576.27</v>
+        <v>23422.75</v>
       </c>
       <c r="C18" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A18</f>
@@ -3179,11 +3179,11 @@
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">B18*C18</f>
-        <v>1390.38356962933</v>
+        <v>20660.5510195179</v>
       </c>
       <c r="E18" s="13" t="n">
         <f aca="false">E17+D18</f>
-        <v>-115489.413732524</v>
+        <v>-70013.4641227035</v>
       </c>
       <c r="F18" s="16" t="str">
         <f aca="false">IF(E18&gt;=0,"Sim","Não")</f>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G13</f>
-        <v>6066.31</v>
+        <v>34039.25</v>
       </c>
       <c r="C19" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A19</f>
@@ -3204,11 +3204,11 @@
       </c>
       <c r="D19" s="12" t="n">
         <f aca="false">B19*C19</f>
-        <v>5255.85622347667</v>
+        <v>29491.6355997267</v>
       </c>
       <c r="E19" s="13" t="n">
         <f aca="false">E18+D19</f>
-        <v>-110233.557509047</v>
+        <v>-40521.8285229768</v>
       </c>
       <c r="F19" s="16" t="str">
         <f aca="false">IF(E19&gt;=0,"Sim","Não")</f>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="B20" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G14</f>
-        <v>5361.84</v>
+        <v>39404.6</v>
       </c>
       <c r="C20" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A20</f>
@@ -3229,11 +3229,11 @@
       </c>
       <c r="D20" s="12" t="n">
         <f aca="false">B20*C20</f>
-        <v>4562.96971591894</v>
+        <v>33533.6370477111</v>
       </c>
       <c r="E20" s="13" t="n">
         <f aca="false">E19+D20</f>
-        <v>-105670.587793128</v>
+        <v>-6988.19147526565</v>
       </c>
       <c r="F20" s="16" t="str">
         <f aca="false">IF(E20&gt;=0,"Sim","Não")</f>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G15</f>
-        <v>9440.55</v>
+        <v>50715.18</v>
       </c>
       <c r="C21" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A21</f>
@@ -3254,15 +3254,15 @@
       </c>
       <c r="D21" s="12" t="n">
         <f aca="false">B21*C21</f>
-        <v>7891.25163710507</v>
+        <v>42392.2596883739</v>
       </c>
       <c r="E21" s="13" t="n">
         <f aca="false">E20+D21</f>
-        <v>-97779.336156023</v>
+        <v>35404.0682131083</v>
       </c>
       <c r="F21" s="16" t="str">
         <f aca="false">IF(E21&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3271,7 +3271,7 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G16</f>
-        <v>8791.43</v>
+        <v>56290.51</v>
       </c>
       <c r="C22" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A22</f>
@@ -3279,15 +3279,15 @@
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">B22*C22</f>
-        <v>7218.10138328468</v>
+        <v>46216.6687440838</v>
       </c>
       <c r="E22" s="13" t="n">
         <f aca="false">E21+D22</f>
-        <v>-90561.2347727383</v>
+        <v>81620.736957192</v>
       </c>
       <c r="F22" s="16" t="str">
         <f aca="false">IF(E22&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="B23" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G17</f>
-        <v>12810.56</v>
+        <v>67388.04</v>
       </c>
       <c r="C23" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A23</f>
@@ -3304,15 +3304,15 @@
       </c>
       <c r="D23" s="12" t="n">
         <f aca="false">B23*C23</f>
-        <v>10331.0967741935</v>
+        <v>54345.1935483871</v>
       </c>
       <c r="E23" s="13" t="n">
         <f aca="false">E22+D23</f>
-        <v>-80230.1379985447</v>
+        <v>135965.930505579</v>
       </c>
       <c r="F23" s="16" t="str">
         <f aca="false">IF(E23&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="B24" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G18</f>
-        <v>16779.05</v>
+        <v>76192.01</v>
       </c>
       <c r="C24" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A24</f>
@@ -3329,15 +3329,15 @@
       </c>
       <c r="D24" s="12" t="n">
         <f aca="false">B24*C24</f>
-        <v>13291.0882799251</v>
+        <v>60353.520082182</v>
       </c>
       <c r="E24" s="13" t="n">
         <f aca="false">E23+D24</f>
-        <v>-66939.0497186196</v>
+        <v>196319.450587761</v>
       </c>
       <c r="F24" s="16" t="str">
         <f aca="false">IF(E24&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="B25" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G19</f>
-        <v>18455.26</v>
+        <v>84540.85</v>
       </c>
       <c r="C25" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A25</f>
@@ -3354,15 +3354,15 @@
       </c>
       <c r="D25" s="12" t="n">
         <f aca="false">B25*C25</f>
-        <v>14359.1324648796</v>
+        <v>65777.0881495853</v>
       </c>
       <c r="E25" s="13" t="n">
         <f aca="false">E24+D25</f>
-        <v>-52579.9172537401</v>
+        <v>262096.538737346</v>
       </c>
       <c r="F25" s="16" t="str">
         <f aca="false">IF(E25&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="B26" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G20</f>
-        <v>21030.24</v>
+        <v>92814.21</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A26</f>
@@ -3379,15 +3379,15 @@
       </c>
       <c r="D26" s="12" t="n">
         <f aca="false">B26*C26</f>
-        <v>16071.8963340678</v>
+        <v>70931.2096033328</v>
       </c>
       <c r="E26" s="13" t="n">
         <f aca="false">E25+D26</f>
-        <v>-36508.0209196723</v>
+        <v>333027.748340679</v>
       </c>
       <c r="F26" s="16" t="str">
         <f aca="false">IF(E26&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="B27" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G21</f>
-        <v>23505.03</v>
+        <v>101840.56</v>
       </c>
       <c r="C27" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A27</f>
@@ -3404,15 +3404,15 @@
       </c>
       <c r="D27" s="12" t="n">
         <f aca="false">B27*C27</f>
-        <v>17644.061502401</v>
+        <v>76446.6628665848</v>
       </c>
       <c r="E27" s="13" t="n">
         <f aca="false">E26+D27</f>
-        <v>-18863.9594172713</v>
+        <v>409474.411207264</v>
       </c>
       <c r="F27" s="16" t="str">
         <f aca="false">IF(E27&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G22</f>
-        <v>25344.17</v>
+        <v>111040.81</v>
       </c>
       <c r="C28" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A28</f>
@@ -3429,15 +3429,15 @@
       </c>
       <c r="D28" s="12" t="n">
         <f aca="false">B28*C28</f>
-        <v>18686.6170558562</v>
+        <v>81871.9687424008</v>
       </c>
       <c r="E28" s="13" t="n">
         <f aca="false">E27+D28</f>
-        <v>-177.34236141506</v>
+        <v>491346.379949665</v>
       </c>
       <c r="F28" s="16" t="str">
         <f aca="false">IF(E28&gt;=0,"Sim","Não")</f>
-        <v>Não</v>
+        <v>Sim</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B29" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G23</f>
-        <v>27936.65</v>
+        <v>121144.29</v>
       </c>
       <c r="C29" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A29</f>
@@ -3454,11 +3454,11 @@
       </c>
       <c r="D29" s="12" t="n">
         <f aca="false">B29*C29</f>
-        <v>20232.138955106</v>
+        <v>87734.5032026983</v>
       </c>
       <c r="E29" s="13" t="n">
         <f aca="false">E28+D29</f>
-        <v>20054.796593691</v>
+        <v>579080.883152363</v>
       </c>
       <c r="F29" s="16" t="str">
         <f aca="false">IF(E29&gt;=0,"Sim","Não")</f>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B30" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G24</f>
-        <v>31346.99</v>
+        <v>130966.8</v>
       </c>
       <c r="C30" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A30</f>
@@ -3479,11 +3479,11 @@
       </c>
       <c r="D30" s="12" t="n">
         <f aca="false">B30*C30</f>
-        <v>22298.6297855344</v>
+        <v>93163.0178015857</v>
       </c>
       <c r="E30" s="13" t="n">
         <f aca="false">E29+D30</f>
-        <v>42353.4263792254</v>
+        <v>672243.900953949</v>
       </c>
       <c r="F30" s="16" t="str">
         <f aca="false">IF(E30&gt;=0,"Sim","Não")</f>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="B31" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G25</f>
-        <v>33939.53</v>
+        <v>143982.38</v>
       </c>
       <c r="C31" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A31</f>
@@ -3504,11 +3504,11 @@
       </c>
       <c r="D31" s="12" t="n">
         <f aca="false">B31*C31</f>
-        <v>23713.9016980633</v>
+        <v>100601.982572334</v>
       </c>
       <c r="E31" s="13" t="n">
         <f aca="false">E30+D31</f>
-        <v>66067.3280772887</v>
+        <v>772845.883526283</v>
       </c>
       <c r="F31" s="16" t="str">
         <f aca="false">IF(E31&gt;=0,"Sim","Não")</f>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="B32" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G26</f>
-        <v>36597.94</v>
+        <v>149241.25</v>
       </c>
       <c r="C32" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A32</f>
@@ -3529,11 +3529,11 @@
       </c>
       <c r="D32" s="12" t="n">
         <f aca="false">B32*C32</f>
-        <v>25117.0535651787</v>
+        <v>102423.810476334</v>
       </c>
       <c r="E32" s="13" t="n">
         <f aca="false">E31+D32</f>
-        <v>91184.3816424674</v>
+        <v>875269.694002616</v>
       </c>
       <c r="F32" s="16" t="str">
         <f aca="false">IF(E32&gt;=0,"Sim","Não")</f>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="B33" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G27</f>
-        <v>38534.55</v>
+        <v>155103.07</v>
       </c>
       <c r="C33" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A33</f>
@@ -3554,11 +3554,11 @@
       </c>
       <c r="D33" s="12" t="n">
         <f aca="false">B33*C33</f>
-        <v>25976.2946743131</v>
+        <v>104555.601433275</v>
       </c>
       <c r="E33" s="13" t="n">
         <f aca="false">E32+D33</f>
-        <v>117160.676316781</v>
+        <v>979825.295435891</v>
       </c>
       <c r="F33" s="16" t="str">
         <f aca="false">IF(E33&gt;=0,"Sim","Não")</f>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B34" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G28</f>
-        <v>39699.21</v>
+        <v>160782.98</v>
       </c>
       <c r="C34" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A34</f>
@@ -3579,11 +3579,11 @@
       </c>
       <c r="D34" s="12" t="n">
         <f aca="false">B34*C34</f>
-        <v>26285.9474085622</v>
+        <v>106458.867984323</v>
       </c>
       <c r="E34" s="13" t="n">
         <f aca="false">E33+D34</f>
-        <v>143446.623725343</v>
+        <v>1086284.16342021</v>
       </c>
       <c r="F34" s="16" t="str">
         <f aca="false">IF(E34&gt;=0,"Sim","Não")</f>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="B35" s="12" t="n">
         <f aca="false">'Fluxo de Caixa'!G29</f>
-        <v>44714.24</v>
+        <v>206907.23</v>
       </c>
       <c r="C35" s="23" t="n">
         <f aca="false">1/(1+$B$7)^A35</f>
@@ -3604,11 +3604,11 @@
       </c>
       <c r="D35" s="12" t="n">
         <f aca="false">B35*C35</f>
-        <v>29080.5411030177</v>
+        <v>134565.055931321</v>
       </c>
       <c r="E35" s="13" t="n">
         <f aca="false">E34+D35</f>
-        <v>172527.16482836</v>
+        <v>1220849.21935154</v>
       </c>
       <c r="F35" s="16" t="str">
         <f aca="false">IF(E35&gt;=0,"Sim","Não")</f>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B38" s="24" t="n">
         <f aca="false">SUM(D11:D35)</f>
-        <v>172527.16482836</v>
+        <v>1220849.21935154</v>
       </c>
       <c r="C38" s="25" t="str">
         <f aca="false">IF(B38&gt;0,"VIÁVEL: o projeto gera mais do que a taxa exigida",IF(B38&lt;0,"INVIÁVEL: o projeto rende menos que a taxa exigida","EQUILÍBRIO: rende exatamente a taxa exigida"))</f>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="B39" s="26" t="n">
         <f aca="false">IFERROR(IRR(B11:B35),"Não calculável")</f>
-        <v>0.0723318571263788</v>
+        <v>0.196259804548004</v>
       </c>
       <c r="C39" s="25" t="str">
         <f aca="false">IF(ISNUMBER(B39),IF(B39&gt;B7,"VIÁVEL: TIR maior que a taxa de desconto","INVIÁVEL: TIR menor ou igual à taxa de desconto"),"Sem TIR: o fluxo precisa ter valores negativos E positivos")</f>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="B40" s="26" t="n">
         <f aca="false">IF(ISNUMBER(B39),IF(B6="Mensal",(1+B39)^12-1,B39),"Não calculável")</f>
-        <v>1.31180127983115</v>
+        <v>7.58827858063135</v>
       </c>
       <c r="C40" s="25" t="str">
         <f aca="false">"Compare com a taxa anual de "&amp;ROUND(B5*100,2)&amp;"%"</f>
@@ -3684,11 +3684,11 @@
       </c>
       <c r="B42" s="26" t="n">
         <f aca="false">IF(B41=0,"-",B38/B41)</f>
-        <v>1.69144279243491</v>
+        <v>11.9691099936425</v>
       </c>
       <c r="C42" s="25" t="str">
         <f aca="false">"Para cada R$ 100 de investimento inicial, o projeto gera R$ "&amp;IF(ISNUMBER(B42),ROUND(B42*100,2),"-")&amp;" de VPL acima da taxa exigida"</f>
-        <v>Para cada R$ 100 de investimento inicial, o projeto gera R$ 169.14 de VPL acima da taxa exigida</v>
+        <v>Para cada R$ 100 de investimento inicial, o projeto gera R$ 1196.91 de VPL acima da taxa exigida</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B43" s="27" t="n">
         <f aca="false">'Necessidade de Caixa e Payback'!F33</f>
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C43" s="25" t="str">
         <f aca="false">"Período em que o saldo acumulado (sem descontar) fica positivo"</f>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="B44" s="27" t="n">
         <f aca="false">IFERROR(INDEX(A11:A35,MATCH("Sim",F11:F35,0)),"Não recupera")</f>
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C44" s="25" t="str">
         <f aca="false">"Período em que o VP acumulado fica positivo"</f>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="B45" s="24" t="n">
         <f aca="false">'Necessidade de Caixa e Payback'!F32</f>
-        <v>120917.64</v>
+        <v>118526.3</v>
       </c>
       <c r="C45" s="25" t="str">
         <f aca="false">"Dinheiro que os sócios precisam ter para cobrir o pior momento"</f>

</xml_diff>